<commit_message>
Fixes for Sagemcom T210-D, minor bugfixes, debug stuff
</commit_message>
<xml_diff>
--- a/data/AuswertungDLMS_ADPU.xlsx
+++ b/data/AuswertungDLMS_ADPU.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24931"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="23231"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Dropbox\WORKSPACE_ESP\___SMARTMETER\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="M:\Dropbox\WORKSPACE_ESP\esp-smartmeter\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7541413C-88FB-4C26-86D2-425CB86E567D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{46C9112D-F8B5-46C2-A8A8-2A7CEA426168}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="3420" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="A" sheetId="1" r:id="rId1"/>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="282" uniqueCount="72">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="794" uniqueCount="144">
   <si>
     <t>'0F</t>
   </si>
@@ -247,13 +247,229 @@
   </si>
   <si>
     <t>XX</t>
+  </si>
+  <si>
+    <t>'0f</t>
+  </si>
+  <si>
+    <t>'0c</t>
+  </si>
+  <si>
+    <t>'e7</t>
+  </si>
+  <si>
+    <t>'0e</t>
+  </si>
+  <si>
+    <t>'ff</t>
+  </si>
+  <si>
+    <t>'88</t>
+  </si>
+  <si>
+    <t>'cc</t>
+  </si>
+  <si>
+    <t>'1e</t>
+  </si>
+  <si>
+    <t>'1b</t>
+  </si>
+  <si>
+    <t>'1f</t>
+  </si>
+  <si>
+    <t>'fe</t>
+  </si>
+  <si>
+    <t>'79</t>
+  </si>
+  <si>
+    <t>'11</t>
+  </si>
+  <si>
+    <t>'38</t>
+  </si>
+  <si>
+    <t>'93</t>
+  </si>
+  <si>
+    <t>'19</t>
+  </si>
+  <si>
+    <t>'3d</t>
+  </si>
+  <si>
+    <t>'44</t>
+  </si>
+  <si>
+    <t>'55</t>
+  </si>
+  <si>
+    <t>'5e</t>
+  </si>
+  <si>
+    <t>Wirkenergie Lieferung [kWh]</t>
+  </si>
+  <si>
+    <t>Wirkenergie Bezug [kWh]</t>
+  </si>
+  <si>
+    <t>Wirkleistung Bezug [kW]</t>
+  </si>
+  <si>
+    <t>Wirkleistung Lieferung [kW]</t>
+  </si>
+  <si>
+    <t>Spannung L1 (V)</t>
+  </si>
+  <si>
+    <t>Spannung L2 (V)</t>
+  </si>
+  <si>
+    <t>Spannung L3 (V)</t>
+  </si>
+  <si>
+    <t>Strom L1  (A)</t>
+  </si>
+  <si>
+    <t>StromL2 (A)</t>
+  </si>
+  <si>
+    <t>'76</t>
+  </si>
+  <si>
+    <t>'0d</t>
+  </si>
+  <si>
+    <t>'fd</t>
+  </si>
+  <si>
+    <t>'31</t>
+  </si>
+  <si>
+    <t>'32</t>
+  </si>
+  <si>
+    <t>'ce</t>
+  </si>
+  <si>
+    <t>'15</t>
+  </si>
+  <si>
+    <t>'91</t>
+  </si>
+  <si>
+    <t>'e6</t>
+  </si>
+  <si>
+    <t>'f4</t>
+  </si>
+  <si>
+    <t>'b1</t>
+  </si>
+  <si>
+    <t>'7c</t>
+  </si>
+  <si>
+    <t>'ba</t>
+  </si>
+  <si>
+    <t>'0b</t>
+  </si>
+  <si>
+    <t>'cb</t>
+  </si>
+  <si>
+    <t>'89</t>
+  </si>
+  <si>
+    <t>'dd</t>
+  </si>
+  <si>
+    <t>'a2</t>
+  </si>
+  <si>
+    <t>'71</t>
+  </si>
+  <si>
+    <t>'a6</t>
+  </si>
+  <si>
+    <t>'52</t>
+  </si>
+  <si>
+    <t>'9d</t>
+  </si>
+  <si>
+    <t>StromL3 (A)</t>
+  </si>
+  <si>
+    <t>Leistungsfaktor [cos(phi)]</t>
+  </si>
+  <si>
+    <t>0F</t>
+  </si>
+  <si>
+    <t>'86</t>
+  </si>
+  <si>
+    <t>'3D</t>
+  </si>
+  <si>
+    <t>'E7</t>
+  </si>
+  <si>
+    <t>'0E</t>
+  </si>
+  <si>
+    <t>'9D</t>
+  </si>
+  <si>
+    <t>'AC</t>
+  </si>
+  <si>
+    <t>'7D</t>
+  </si>
+  <si>
+    <t>'27</t>
+  </si>
+  <si>
+    <t>'2D</t>
+  </si>
+  <si>
+    <t>'B3</t>
+  </si>
+  <si>
+    <t>'85</t>
+  </si>
+  <si>
+    <t>'CF</t>
+  </si>
+  <si>
+    <t>'17</t>
+  </si>
+  <si>
+    <t>'8B</t>
+  </si>
+  <si>
+    <t>'F4</t>
+  </si>
+  <si>
+    <t>'30</t>
+  </si>
+  <si>
+    <t>'36</t>
+  </si>
+  <si>
+    <t>Trash Data from Sagemcom?????????</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="20" x14ac:knownFonts="1">
+  <fonts count="21" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -403,8 +619,16 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="8"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="41">
+  <fills count="42">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -632,8 +856,14 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF0000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="32">
+  <borders count="33">
     <border>
       <left/>
       <right/>
@@ -1002,6 +1232,15 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="50">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -1055,7 +1294,7 @@
     <xf numFmtId="2" fontId="18" fillId="39" borderId="15" applyFont="0"/>
     <xf numFmtId="2" fontId="18" fillId="40" borderId="15"/>
   </cellStyleXfs>
-  <cellXfs count="85">
+  <cellXfs count="91">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1124,7 +1363,6 @@
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" textRotation="90"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="3" borderId="26" xfId="7" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="3" borderId="27" xfId="7" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="3" borderId="28" xfId="7" applyBorder="1"/>
@@ -1134,12 +1372,21 @@
     <xf numFmtId="2" fontId="18" fillId="40" borderId="10" xfId="49" applyBorder="1"/>
     <xf numFmtId="2" fontId="18" fillId="40" borderId="11" xfId="49" applyBorder="1"/>
     <xf numFmtId="2" fontId="18" fillId="40" borderId="12" xfId="49" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="31" xfId="0" applyBorder="1"/>
     <xf numFmtId="2" fontId="18" fillId="39" borderId="17" xfId="48" applyFont="1" applyBorder="1"/>
     <xf numFmtId="2" fontId="18" fillId="39" borderId="18" xfId="48" applyFont="1" applyBorder="1"/>
     <xf numFmtId="2" fontId="18" fillId="40" borderId="16" xfId="49" applyBorder="1"/>
     <xf numFmtId="2" fontId="0" fillId="39" borderId="17" xfId="48" applyFont="1" applyBorder="1"/>
     <xf numFmtId="2" fontId="0" fillId="39" borderId="18" xfId="48" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1170,14 +1417,18 @@
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" textRotation="90"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="30" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
+    <xf numFmtId="0" fontId="16" fillId="41" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="50">
@@ -1550,7 +1801,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:IJ22"/>
+  <dimension ref="A1:IX26"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5.5703125" style="18" bestFit="1" customWidth="1"/>
@@ -1573,30 +1824,264 @@
     <col min="92" max="92" width="3.7109375" bestFit="1" customWidth="1"/>
     <col min="93" max="100" width="3.5703125" bestFit="1" customWidth="1"/>
     <col min="101" max="244" width="4" bestFit="1" customWidth="1"/>
+    <col min="245" max="258" width="3.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:244" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="X1" s="82">
+    <row r="1" spans="1:258" s="74" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="70"/>
+      <c r="B1" s="71"/>
+      <c r="C1" s="71"/>
+      <c r="D1" s="71"/>
+      <c r="E1" s="71"/>
+      <c r="F1" s="71"/>
+      <c r="G1" s="71"/>
+      <c r="H1" s="71"/>
+      <c r="I1" s="71"/>
+      <c r="J1" s="71"/>
+      <c r="K1" s="71"/>
+      <c r="L1" s="71"/>
+      <c r="M1" s="71"/>
+      <c r="N1" s="71"/>
+      <c r="O1" s="71"/>
+      <c r="P1" s="71"/>
+      <c r="Q1" s="71"/>
+      <c r="R1" s="71"/>
+      <c r="S1" s="71"/>
+      <c r="T1" s="71"/>
+      <c r="U1" s="71"/>
+      <c r="V1" s="71"/>
+      <c r="W1" s="71"/>
+      <c r="X1" s="86">
         <v>2022</v>
       </c>
-      <c r="Y1" s="83"/>
-      <c r="Z1" s="66">
+      <c r="Y1" s="87"/>
+      <c r="Z1" s="72">
         <v>2</v>
       </c>
-      <c r="AA1" s="66">
+      <c r="AA1" s="72">
         <v>4</v>
       </c>
-      <c r="AC1" s="66">
+      <c r="AB1" s="71"/>
+      <c r="AC1" s="72">
         <v>16</v>
       </c>
-      <c r="AD1" s="66">
+      <c r="AD1" s="72">
         <v>43</v>
       </c>
-      <c r="AE1" s="56">
+      <c r="AE1" s="73">
         <v>20</v>
       </c>
+      <c r="AF1" s="71"/>
+      <c r="AG1" s="71"/>
+      <c r="AH1" s="71"/>
+      <c r="AI1" s="71"/>
+      <c r="AJ1" s="71"/>
+      <c r="AK1" s="71"/>
+      <c r="AL1" s="75" t="s">
+        <v>93</v>
+      </c>
+      <c r="AM1" s="75"/>
+      <c r="AN1" s="75"/>
+      <c r="AO1" s="75"/>
+      <c r="AP1" s="75"/>
+      <c r="AQ1" s="75"/>
+      <c r="AR1" s="71"/>
+      <c r="AS1" s="71"/>
+      <c r="AT1" s="71"/>
+      <c r="AU1" s="71"/>
+      <c r="AV1" s="71"/>
+      <c r="AW1" s="71"/>
+      <c r="AX1" s="71"/>
+      <c r="AY1" s="71"/>
+      <c r="AZ1" s="71"/>
+      <c r="BA1" s="71"/>
+      <c r="BB1" s="71"/>
+      <c r="BC1" s="71"/>
+      <c r="BD1" s="71"/>
+      <c r="BE1" s="75" t="s">
+        <v>92</v>
+      </c>
+      <c r="BF1" s="75"/>
+      <c r="BG1" s="75"/>
+      <c r="BH1" s="75"/>
+      <c r="BI1" s="75"/>
+      <c r="BJ1" s="75"/>
+      <c r="BK1" s="71"/>
+      <c r="BL1" s="71"/>
+      <c r="BM1" s="71"/>
+      <c r="BN1" s="71"/>
+      <c r="BO1" s="71"/>
+      <c r="BP1" s="71"/>
+      <c r="BQ1" s="71"/>
+      <c r="BR1" s="71"/>
+      <c r="BS1" s="71"/>
+      <c r="BT1" s="71"/>
+      <c r="BU1" s="71"/>
+      <c r="BV1" s="71"/>
+      <c r="BW1" s="71"/>
+      <c r="BX1" s="75" t="s">
+        <v>94</v>
+      </c>
+      <c r="BY1" s="75"/>
+      <c r="BZ1" s="75"/>
+      <c r="CA1" s="75"/>
+      <c r="CB1" s="75"/>
+      <c r="CC1" s="75"/>
+      <c r="CD1" s="71"/>
+      <c r="CE1" s="71"/>
+      <c r="CF1" s="71"/>
+      <c r="CG1" s="71"/>
+      <c r="CH1" s="71"/>
+      <c r="CI1" s="71"/>
+      <c r="CJ1" s="71"/>
+      <c r="CK1" s="71"/>
+      <c r="CL1" s="71"/>
+      <c r="CM1" s="71"/>
+      <c r="CN1" s="71"/>
+      <c r="CO1" s="71"/>
+      <c r="CP1" s="71"/>
+      <c r="CQ1" s="75" t="s">
+        <v>95</v>
+      </c>
+      <c r="CR1" s="75"/>
+      <c r="CS1" s="75"/>
+      <c r="CT1" s="75"/>
+      <c r="CU1" s="75"/>
+      <c r="CV1" s="75"/>
+      <c r="CW1" s="71"/>
+      <c r="CX1" s="71"/>
+      <c r="CY1" s="71"/>
+      <c r="CZ1" s="71"/>
+      <c r="DA1" s="71"/>
+      <c r="DB1" s="71"/>
+      <c r="DC1" s="71"/>
+      <c r="DD1" s="71"/>
+      <c r="DE1" s="71"/>
+      <c r="DF1" s="71"/>
+      <c r="DG1" s="71"/>
+      <c r="DH1" s="71"/>
+      <c r="DI1" s="71"/>
+      <c r="DJ1" s="75" t="s">
+        <v>96</v>
+      </c>
+      <c r="DK1" s="75"/>
+      <c r="DL1" s="75"/>
+      <c r="DM1" s="75"/>
+      <c r="DN1" s="75"/>
+      <c r="DO1" s="75"/>
+      <c r="DP1" s="71"/>
+      <c r="DQ1" s="71"/>
+      <c r="DR1" s="71"/>
+      <c r="DS1" s="71"/>
+      <c r="DT1" s="71"/>
+      <c r="DU1" s="71"/>
+      <c r="DV1" s="71"/>
+      <c r="DW1" s="71"/>
+      <c r="DX1" s="71"/>
+      <c r="DY1" s="71"/>
+      <c r="DZ1" s="71"/>
+      <c r="EA1" s="75" t="s">
+        <v>97</v>
+      </c>
+      <c r="EB1" s="75"/>
+      <c r="EC1" s="75"/>
+      <c r="ED1" s="75"/>
+      <c r="EE1" s="75"/>
+      <c r="EF1" s="75"/>
+      <c r="EG1" s="71"/>
+      <c r="EH1" s="71"/>
+      <c r="EI1" s="71"/>
+      <c r="EJ1" s="71"/>
+      <c r="EK1" s="71"/>
+      <c r="EL1" s="71"/>
+      <c r="EM1" s="71"/>
+      <c r="EN1" s="71"/>
+      <c r="EO1" s="71"/>
+      <c r="EP1" s="71"/>
+      <c r="EQ1" s="71"/>
+      <c r="ER1" s="75" t="s">
+        <v>98</v>
+      </c>
+      <c r="ES1" s="75"/>
+      <c r="ET1" s="75"/>
+      <c r="EU1" s="75"/>
+      <c r="EV1" s="75"/>
+      <c r="EW1" s="75"/>
+      <c r="EX1" s="71"/>
+      <c r="EY1" s="71"/>
+      <c r="EZ1" s="71"/>
+      <c r="FA1" s="71"/>
+      <c r="FB1" s="71"/>
+      <c r="FC1" s="71"/>
+      <c r="FD1" s="71"/>
+      <c r="FE1" s="71"/>
+      <c r="FF1" s="71"/>
+      <c r="FG1" s="71"/>
+      <c r="FH1" s="71"/>
+      <c r="FI1" s="75" t="s">
+        <v>99</v>
+      </c>
+      <c r="FJ1" s="75"/>
+      <c r="FK1" s="75"/>
+      <c r="FL1" s="75"/>
+      <c r="FM1" s="75"/>
+      <c r="FN1" s="75"/>
+      <c r="FO1" s="71"/>
+      <c r="FP1" s="71"/>
+      <c r="FQ1" s="71"/>
+      <c r="FR1" s="71"/>
+      <c r="FS1" s="71"/>
+      <c r="FT1" s="71"/>
+      <c r="FU1" s="71"/>
+      <c r="FV1" s="71"/>
+      <c r="FW1" s="71"/>
+      <c r="FX1" s="71"/>
+      <c r="FY1" s="71"/>
+      <c r="FZ1" s="75" t="s">
+        <v>100</v>
+      </c>
+      <c r="GA1" s="75"/>
+      <c r="GB1" s="75"/>
+      <c r="GC1" s="75"/>
+      <c r="GD1" s="75"/>
+      <c r="GE1" s="75"/>
+      <c r="GF1" s="71"/>
+      <c r="GG1" s="71"/>
+      <c r="GH1" s="71"/>
+      <c r="GI1" s="71"/>
+      <c r="GJ1" s="71"/>
+      <c r="GQ1" s="75" t="s">
+        <v>123</v>
+      </c>
+      <c r="GR1" s="75"/>
+      <c r="GS1" s="75"/>
+      <c r="GT1" s="75"/>
+      <c r="GU1" s="75"/>
+      <c r="GV1" s="75"/>
+      <c r="HH1" s="75" t="s">
+        <v>124</v>
+      </c>
+      <c r="HI1" s="75"/>
+      <c r="HJ1" s="75"/>
+      <c r="HK1" s="75"/>
+      <c r="HL1" s="75"/>
+      <c r="HM1" s="75"/>
+      <c r="HY1" s="75" t="s">
+        <v>45</v>
+      </c>
+      <c r="HZ1" s="75"/>
+      <c r="IA1" s="75"/>
+      <c r="IB1" s="75"/>
+      <c r="IC1" s="75"/>
+      <c r="ID1" s="75"/>
+      <c r="IE1" s="75"/>
+      <c r="IF1" s="75"/>
+      <c r="IG1" s="75"/>
+      <c r="IH1" s="75"/>
+      <c r="II1" s="75"/>
+      <c r="IJ1" s="75"/>
     </row>
-    <row r="2" spans="1:244" s="2" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:258" s="2" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="41" t="s">
         <v>51</v>
       </c>
@@ -1741,13 +2226,13 @@
       <c r="AV2" s="11" t="s">
         <v>12</v>
       </c>
-      <c r="AW2" s="67" t="s">
-        <v>8</v>
-      </c>
-      <c r="AX2" s="68" t="s">
-        <v>8</v>
-      </c>
-      <c r="AY2" s="69" t="s">
+      <c r="AW2" s="65" t="s">
+        <v>8</v>
+      </c>
+      <c r="AX2" s="66" t="s">
+        <v>8</v>
+      </c>
+      <c r="AY2" s="67" t="s">
         <v>0</v>
       </c>
       <c r="AZ2" s="46" t="s">
@@ -1798,13 +2283,13 @@
       <c r="BO2" s="11" t="s">
         <v>13</v>
       </c>
-      <c r="BP2" s="67" t="s">
-        <v>8</v>
-      </c>
-      <c r="BQ2" s="68" t="s">
-        <v>8</v>
-      </c>
-      <c r="BR2" s="69" t="s">
+      <c r="BP2" s="65" t="s">
+        <v>8</v>
+      </c>
+      <c r="BQ2" s="66" t="s">
+        <v>8</v>
+      </c>
+      <c r="BR2" s="67" t="s">
         <v>0</v>
       </c>
       <c r="BS2" s="46" t="s">
@@ -1855,13 +2340,13 @@
       <c r="CH2" s="11" t="s">
         <v>24</v>
       </c>
-      <c r="CI2" s="67" t="s">
-        <v>8</v>
-      </c>
-      <c r="CJ2" s="68" t="s">
-        <v>8</v>
-      </c>
-      <c r="CK2" s="69" t="s">
+      <c r="CI2" s="65" t="s">
+        <v>8</v>
+      </c>
+      <c r="CJ2" s="66" t="s">
+        <v>8</v>
+      </c>
+      <c r="CK2" s="67" t="s">
         <v>0</v>
       </c>
       <c r="CL2" s="46" t="s">
@@ -1912,13 +2397,13 @@
       <c r="DA2" s="11" t="s">
         <v>13</v>
       </c>
-      <c r="DB2" s="67" t="s">
-        <v>8</v>
-      </c>
-      <c r="DC2" s="68" t="s">
-        <v>8</v>
-      </c>
-      <c r="DD2" s="69" t="s">
+      <c r="DB2" s="65" t="s">
+        <v>8</v>
+      </c>
+      <c r="DC2" s="66" t="s">
+        <v>8</v>
+      </c>
+      <c r="DD2" s="67" t="s">
         <v>0</v>
       </c>
       <c r="DE2" s="46" t="s">
@@ -1963,13 +2448,13 @@
       <c r="DR2" s="11" t="s">
         <v>28</v>
       </c>
-      <c r="DS2" s="70" t="s">
-        <v>8</v>
-      </c>
-      <c r="DT2" s="71" t="s">
-        <v>8</v>
-      </c>
-      <c r="DU2" s="69" t="s">
+      <c r="DS2" s="68" t="s">
+        <v>8</v>
+      </c>
+      <c r="DT2" s="69" t="s">
+        <v>8</v>
+      </c>
+      <c r="DU2" s="67" t="s">
         <v>0</v>
       </c>
       <c r="DV2" s="46" t="s">
@@ -2014,13 +2499,13 @@
       <c r="EI2" s="11" t="s">
         <v>23</v>
       </c>
-      <c r="EJ2" s="67" t="s">
-        <v>8</v>
-      </c>
-      <c r="EK2" s="68" t="s">
-        <v>8</v>
-      </c>
-      <c r="EL2" s="69" t="s">
+      <c r="EJ2" s="65" t="s">
+        <v>8</v>
+      </c>
+      <c r="EK2" s="66" t="s">
+        <v>8</v>
+      </c>
+      <c r="EL2" s="67" t="s">
         <v>0</v>
       </c>
       <c r="EM2" s="46" t="s">
@@ -2065,13 +2550,13 @@
       <c r="EZ2" s="11" t="s">
         <v>31</v>
       </c>
-      <c r="FA2" s="67" t="s">
-        <v>8</v>
-      </c>
-      <c r="FB2" s="68" t="s">
-        <v>8</v>
-      </c>
-      <c r="FC2" s="69" t="s">
+      <c r="FA2" s="65" t="s">
+        <v>8</v>
+      </c>
+      <c r="FB2" s="66" t="s">
+        <v>8</v>
+      </c>
+      <c r="FC2" s="67" t="s">
         <v>0</v>
       </c>
       <c r="FD2" s="46" t="s">
@@ -2116,13 +2601,13 @@
       <c r="FQ2" s="11" t="s">
         <v>32</v>
       </c>
-      <c r="FR2" s="67" t="s">
-        <v>8</v>
-      </c>
-      <c r="FS2" s="68" t="s">
-        <v>8</v>
-      </c>
-      <c r="FT2" s="69" t="s">
+      <c r="FR2" s="65" t="s">
+        <v>8</v>
+      </c>
+      <c r="FS2" s="66" t="s">
+        <v>8</v>
+      </c>
+      <c r="FT2" s="67" t="s">
         <v>0</v>
       </c>
       <c r="FU2" s="46" t="s">
@@ -2167,13 +2652,13 @@
       <c r="GH2" s="11" t="s">
         <v>35</v>
       </c>
-      <c r="GI2" s="67" t="s">
-        <v>8</v>
-      </c>
-      <c r="GJ2" s="68" t="s">
-        <v>8</v>
-      </c>
-      <c r="GK2" s="69" t="s">
+      <c r="GI2" s="65" t="s">
+        <v>8</v>
+      </c>
+      <c r="GJ2" s="66" t="s">
+        <v>8</v>
+      </c>
+      <c r="GK2" s="67" t="s">
         <v>0</v>
       </c>
       <c r="GL2" s="46" t="s">
@@ -2218,13 +2703,13 @@
       <c r="GY2" s="11" t="s">
         <v>37</v>
       </c>
-      <c r="GZ2" s="67" t="s">
-        <v>8</v>
-      </c>
-      <c r="HA2" s="68" t="s">
-        <v>8</v>
-      </c>
-      <c r="HB2" s="69" t="s">
+      <c r="GZ2" s="65" t="s">
+        <v>8</v>
+      </c>
+      <c r="HA2" s="66" t="s">
+        <v>8</v>
+      </c>
+      <c r="HB2" s="67" t="s">
         <v>0</v>
       </c>
       <c r="HC2" s="46" t="s">
@@ -2269,13 +2754,13 @@
       <c r="HP2" s="11" t="s">
         <v>40</v>
       </c>
-      <c r="HQ2" s="67" t="s">
-        <v>8</v>
-      </c>
-      <c r="HR2" s="68" t="s">
-        <v>8</v>
-      </c>
-      <c r="HS2" s="69" t="s">
+      <c r="HQ2" s="65" t="s">
+        <v>8</v>
+      </c>
+      <c r="HR2" s="66" t="s">
+        <v>8</v>
+      </c>
+      <c r="HS2" s="67" t="s">
         <v>0</v>
       </c>
       <c r="HT2" s="46" t="s">
@@ -2330,1592 +2815,3102 @@
         <v>42</v>
       </c>
     </row>
-    <row r="3" spans="1:244" s="1" customFormat="1" ht="12" x14ac:dyDescent="0.2">
-      <c r="A3" s="1" t="s">
+    <row r="3" spans="1:258" x14ac:dyDescent="0.25">
+      <c r="A3"/>
+    </row>
+    <row r="4" spans="1:258" x14ac:dyDescent="0.25">
+      <c r="A4"/>
+      <c r="HV4" s="90" t="s">
+        <v>143</v>
+      </c>
+      <c r="HW4" s="90"/>
+      <c r="HX4" s="90"/>
+      <c r="HY4" s="90"/>
+      <c r="HZ4" s="90"/>
+      <c r="IA4" s="90"/>
+      <c r="IB4" s="90"/>
+      <c r="IC4" s="90"/>
+      <c r="ID4" s="90"/>
+      <c r="IE4" s="90"/>
+      <c r="IF4" s="90"/>
+      <c r="IG4" s="90"/>
+      <c r="IH4" s="90"/>
+      <c r="II4" s="90"/>
+      <c r="IJ4" s="90"/>
+      <c r="IK4" s="90"/>
+      <c r="IL4" s="90"/>
+      <c r="IM4" s="90"/>
+      <c r="IN4" s="90"/>
+      <c r="IO4" s="90"/>
+      <c r="IP4" s="90"/>
+      <c r="IQ4" s="90"/>
+      <c r="IR4" s="90"/>
+      <c r="IS4" s="90"/>
+      <c r="IT4" s="90"/>
+      <c r="IU4" s="90"/>
+      <c r="IV4" s="90"/>
+      <c r="IW4" s="90"/>
+      <c r="IX4" s="90"/>
+    </row>
+    <row r="5" spans="1:258" x14ac:dyDescent="0.25">
+      <c r="A5"/>
+      <c r="B5" s="89" t="s">
+        <v>125</v>
+      </c>
+      <c r="C5" t="s">
+        <v>1</v>
+      </c>
+      <c r="D5" t="s">
+        <v>13</v>
+      </c>
+      <c r="E5" t="s">
+        <v>126</v>
+      </c>
+      <c r="F5" t="s">
+        <v>127</v>
+      </c>
+      <c r="G5" t="s">
+        <v>5</v>
+      </c>
+      <c r="H5" t="s">
+        <v>6</v>
+      </c>
+      <c r="I5" t="s">
+        <v>128</v>
+      </c>
+      <c r="J5" t="s">
+        <v>4</v>
+      </c>
+      <c r="K5" t="s">
+        <v>129</v>
+      </c>
+      <c r="L5" t="s">
+        <v>9</v>
+      </c>
+      <c r="M5" t="s">
+        <v>12</v>
+      </c>
+      <c r="N5" t="s">
+        <v>13</v>
+      </c>
+      <c r="O5" t="s">
+        <v>9</v>
+      </c>
+      <c r="P5" t="s">
+        <v>13</v>
+      </c>
+      <c r="Q5" t="s">
+        <v>14</v>
+      </c>
+      <c r="R5" t="s">
+        <v>77</v>
+      </c>
+      <c r="S5" t="s">
+        <v>1</v>
+      </c>
+      <c r="T5" t="s">
+        <v>8</v>
+      </c>
+      <c r="U5" t="s">
+        <v>16</v>
+      </c>
+      <c r="V5" t="s">
+        <v>17</v>
+      </c>
+      <c r="W5" t="s">
+        <v>5</v>
+      </c>
+      <c r="X5" t="s">
+        <v>6</v>
+      </c>
+      <c r="Y5" t="s">
+        <v>128</v>
+      </c>
+      <c r="Z5" t="s">
+        <v>4</v>
+      </c>
+      <c r="AA5" t="s">
+        <v>129</v>
+      </c>
+      <c r="AB5" t="s">
+        <v>9</v>
+      </c>
+      <c r="AC5" t="s">
+        <v>12</v>
+      </c>
+      <c r="AD5" t="s">
+        <v>13</v>
+      </c>
+      <c r="AE5" t="s">
+        <v>9</v>
+      </c>
+      <c r="AF5" t="s">
+        <v>13</v>
+      </c>
+      <c r="AG5" t="s">
+        <v>14</v>
+      </c>
+      <c r="AH5" t="s">
+        <v>77</v>
+      </c>
+      <c r="AI5" t="s">
+        <v>1</v>
+      </c>
+      <c r="AJ5" t="s">
+        <v>17</v>
+      </c>
+      <c r="AK5" t="s">
+        <v>18</v>
+      </c>
+      <c r="AL5" t="s">
+        <v>19</v>
+      </c>
+      <c r="AM5" t="s">
+        <v>13</v>
+      </c>
+      <c r="AN5" t="s">
+        <v>19</v>
+      </c>
+      <c r="AO5" t="s">
+        <v>20</v>
+      </c>
+      <c r="AP5" t="s">
+        <v>13</v>
+      </c>
+      <c r="AQ5" t="s">
+        <v>14</v>
+      </c>
+      <c r="AR5" t="s">
+        <v>18</v>
+      </c>
+      <c r="AS5" t="s">
+        <v>13</v>
+      </c>
+      <c r="AT5" t="s">
+        <v>17</v>
+      </c>
+      <c r="AU5" t="s">
+        <v>130</v>
+      </c>
+      <c r="AV5" t="s">
+        <v>131</v>
+      </c>
+      <c r="AW5" t="s">
+        <v>8</v>
+      </c>
+      <c r="AX5" t="s">
+        <v>8</v>
+      </c>
+      <c r="AY5" t="s">
+        <v>0</v>
+      </c>
+      <c r="AZ5" t="s">
+        <v>13</v>
+      </c>
+      <c r="BA5" t="s">
+        <v>22</v>
+      </c>
+      <c r="BB5" t="s">
+        <v>23</v>
+      </c>
+      <c r="BC5" t="s">
+        <v>17</v>
+      </c>
+      <c r="BD5" t="s">
+        <v>18</v>
+      </c>
+      <c r="BE5" t="s">
+        <v>19</v>
+      </c>
+      <c r="BF5" t="s">
+        <v>13</v>
+      </c>
+      <c r="BG5" t="s">
+        <v>8</v>
+      </c>
+      <c r="BH5" t="s">
+        <v>20</v>
+      </c>
+      <c r="BI5" t="s">
+        <v>13</v>
+      </c>
+      <c r="BJ5" t="s">
+        <v>14</v>
+      </c>
+      <c r="BK5" t="s">
+        <v>18</v>
+      </c>
+      <c r="BL5" t="s">
+        <v>13</v>
+      </c>
+      <c r="BM5" t="s">
+        <v>13</v>
+      </c>
+      <c r="BN5" t="s">
+        <v>13</v>
+      </c>
+      <c r="BO5" t="s">
+        <v>13</v>
+      </c>
+      <c r="BP5" t="s">
+        <v>8</v>
+      </c>
+      <c r="BQ5" t="s">
+        <v>8</v>
+      </c>
+      <c r="BR5" t="s">
+        <v>0</v>
+      </c>
+      <c r="BS5" t="s">
+        <v>13</v>
+      </c>
+      <c r="BT5" t="s">
+        <v>22</v>
+      </c>
+      <c r="BU5" t="s">
+        <v>23</v>
+      </c>
+      <c r="BV5" t="s">
+        <v>17</v>
+      </c>
+      <c r="BW5" t="s">
+        <v>18</v>
+      </c>
+      <c r="BX5" t="s">
+        <v>19</v>
+      </c>
+      <c r="BY5" t="s">
+        <v>13</v>
+      </c>
+      <c r="BZ5" t="s">
+        <v>19</v>
+      </c>
+      <c r="CA5" t="s">
+        <v>6</v>
+      </c>
+      <c r="CB5" t="s">
+        <v>13</v>
+      </c>
+      <c r="CC5" t="s">
+        <v>14</v>
+      </c>
+      <c r="CD5" t="s">
+        <v>18</v>
+      </c>
+      <c r="CE5" t="s">
+        <v>13</v>
+      </c>
+      <c r="CF5" t="s">
+        <v>13</v>
+      </c>
+      <c r="CG5" t="s">
+        <v>39</v>
+      </c>
+      <c r="CH5" t="s">
+        <v>132</v>
+      </c>
+      <c r="CI5" t="s">
+        <v>8</v>
+      </c>
+      <c r="CJ5" t="s">
+        <v>8</v>
+      </c>
+      <c r="CK5" t="s">
+        <v>0</v>
+      </c>
+      <c r="CL5" t="s">
+        <v>13</v>
+      </c>
+      <c r="CM5" t="s">
+        <v>22</v>
+      </c>
+      <c r="CN5" t="s">
+        <v>25</v>
+      </c>
+      <c r="CO5" t="s">
+        <v>17</v>
+      </c>
+      <c r="CP5" t="s">
+        <v>18</v>
+      </c>
+      <c r="CQ5" t="s">
+        <v>19</v>
+      </c>
+      <c r="CR5" t="s">
+        <v>13</v>
+      </c>
+      <c r="CS5" t="s">
+        <v>8</v>
+      </c>
+      <c r="CT5" t="s">
+        <v>6</v>
+      </c>
+      <c r="CU5" t="s">
+        <v>13</v>
+      </c>
+      <c r="CV5" t="s">
+        <v>14</v>
+      </c>
+      <c r="CW5" t="s">
+        <v>18</v>
+      </c>
+      <c r="CX5" t="s">
+        <v>13</v>
+      </c>
+      <c r="CY5" t="s">
+        <v>13</v>
+      </c>
+      <c r="CZ5" t="s">
+        <v>13</v>
+      </c>
+      <c r="DA5" t="s">
+        <v>13</v>
+      </c>
+      <c r="DB5" t="s">
+        <v>8</v>
+      </c>
+      <c r="DC5" t="s">
+        <v>8</v>
+      </c>
+      <c r="DD5" t="s">
+        <v>0</v>
+      </c>
+      <c r="DE5" t="s">
+        <v>13</v>
+      </c>
+      <c r="DF5" t="s">
+        <v>22</v>
+      </c>
+      <c r="DG5" t="s">
+        <v>25</v>
+      </c>
+      <c r="DH5" t="s">
+        <v>17</v>
+      </c>
+      <c r="DI5" t="s">
+        <v>18</v>
+      </c>
+      <c r="DJ5" t="s">
+        <v>19</v>
+      </c>
+      <c r="DK5" t="s">
+        <v>13</v>
+      </c>
+      <c r="DL5" t="s">
+        <v>26</v>
+      </c>
+      <c r="DM5" t="s">
+        <v>6</v>
+      </c>
+      <c r="DN5" t="s">
+        <v>13</v>
+      </c>
+      <c r="DO5" t="s">
+        <v>14</v>
+      </c>
+      <c r="DP5" t="s">
+        <v>27</v>
+      </c>
+      <c r="DQ5" t="s">
+        <v>17</v>
+      </c>
+      <c r="DR5" t="s">
+        <v>133</v>
+      </c>
+      <c r="DS5" t="s">
+        <v>8</v>
+      </c>
+      <c r="DT5" t="s">
+        <v>8</v>
+      </c>
+      <c r="DU5" t="s">
+        <v>0</v>
+      </c>
+      <c r="DV5" t="s">
+        <v>14</v>
+      </c>
+      <c r="DW5" t="s">
+        <v>22</v>
+      </c>
+      <c r="DX5" t="s">
+        <v>16</v>
+      </c>
+      <c r="DY5" t="s">
+        <v>17</v>
+      </c>
+      <c r="DZ5" t="s">
+        <v>18</v>
+      </c>
+      <c r="EA5" t="s">
+        <v>19</v>
+      </c>
+      <c r="EB5" t="s">
+        <v>13</v>
+      </c>
+      <c r="EC5" t="s">
+        <v>29</v>
+      </c>
+      <c r="ED5" t="s">
+        <v>6</v>
+      </c>
+      <c r="EE5" t="s">
+        <v>13</v>
+      </c>
+      <c r="EF5" t="s">
+        <v>14</v>
+      </c>
+      <c r="EG5" t="s">
+        <v>27</v>
+      </c>
+      <c r="EH5" t="s">
+        <v>17</v>
+      </c>
+      <c r="EI5" t="s">
+        <v>87</v>
+      </c>
+      <c r="EJ5" t="s">
+        <v>8</v>
+      </c>
+      <c r="EK5" t="s">
+        <v>8</v>
+      </c>
+      <c r="EL5" t="s">
+        <v>0</v>
+      </c>
+      <c r="EM5" t="s">
+        <v>14</v>
+      </c>
+      <c r="EN5" t="s">
+        <v>22</v>
+      </c>
+      <c r="EO5" t="s">
+        <v>16</v>
+      </c>
+      <c r="EP5" t="s">
+        <v>17</v>
+      </c>
+      <c r="EQ5" t="s">
+        <v>18</v>
+      </c>
+      <c r="ER5" t="s">
+        <v>19</v>
+      </c>
+      <c r="ES5" t="s">
+        <v>13</v>
+      </c>
+      <c r="ET5" t="s">
+        <v>30</v>
+      </c>
+      <c r="EU5" t="s">
+        <v>6</v>
+      </c>
+      <c r="EV5" t="s">
+        <v>13</v>
+      </c>
+      <c r="EW5" t="s">
+        <v>14</v>
+      </c>
+      <c r="EX5" t="s">
+        <v>27</v>
+      </c>
+      <c r="EY5" t="s">
+        <v>17</v>
+      </c>
+      <c r="EZ5" t="s">
+        <v>134</v>
+      </c>
+      <c r="FA5" t="s">
+        <v>8</v>
+      </c>
+      <c r="FB5" t="s">
+        <v>8</v>
+      </c>
+      <c r="FC5" t="s">
+        <v>0</v>
+      </c>
+      <c r="FD5" t="s">
+        <v>14</v>
+      </c>
+      <c r="FE5" t="s">
+        <v>22</v>
+      </c>
+      <c r="FF5" t="s">
+        <v>16</v>
+      </c>
+      <c r="FG5" t="s">
+        <v>17</v>
+      </c>
+      <c r="FH5" t="s">
+        <v>18</v>
+      </c>
+      <c r="FI5" t="s">
+        <v>19</v>
+      </c>
+      <c r="FJ5" t="s">
+        <v>13</v>
+      </c>
+      <c r="FK5" t="s">
+        <v>24</v>
+      </c>
+      <c r="FL5" t="s">
+        <v>6</v>
+      </c>
+      <c r="FM5" t="s">
+        <v>13</v>
+      </c>
+      <c r="FN5" t="s">
+        <v>14</v>
+      </c>
+      <c r="FO5" t="s">
+        <v>27</v>
+      </c>
+      <c r="FP5" t="s">
+        <v>13</v>
+      </c>
+      <c r="FQ5" t="s">
+        <v>135</v>
+      </c>
+      <c r="FR5" t="s">
+        <v>8</v>
+      </c>
+      <c r="FS5" t="s">
+        <v>8</v>
+      </c>
+      <c r="FT5" t="s">
+        <v>0</v>
+      </c>
+      <c r="FU5" t="s">
+        <v>33</v>
+      </c>
+      <c r="FV5" t="s">
+        <v>22</v>
+      </c>
+      <c r="FW5" t="s">
+        <v>31</v>
+      </c>
+      <c r="FX5" t="s">
+        <v>17</v>
+      </c>
+      <c r="FY5" t="s">
+        <v>18</v>
+      </c>
+      <c r="FZ5" t="s">
+        <v>19</v>
+      </c>
+      <c r="GA5" t="s">
+        <v>13</v>
+      </c>
+      <c r="GB5" t="s">
+        <v>34</v>
+      </c>
+      <c r="GC5" t="s">
+        <v>6</v>
+      </c>
+      <c r="GD5" t="s">
+        <v>13</v>
+      </c>
+      <c r="GE5" t="s">
+        <v>14</v>
+      </c>
+      <c r="GF5" t="s">
+        <v>27</v>
+      </c>
+      <c r="GG5" t="s">
+        <v>13</v>
+      </c>
+      <c r="GH5" t="s">
+        <v>35</v>
+      </c>
+      <c r="GI5" t="s">
+        <v>8</v>
+      </c>
+      <c r="GJ5" t="s">
+        <v>8</v>
+      </c>
+      <c r="GK5" t="s">
+        <v>0</v>
+      </c>
+      <c r="GL5" t="s">
+        <v>33</v>
+      </c>
+      <c r="GM5" t="s">
+        <v>22</v>
+      </c>
+      <c r="GN5" t="s">
+        <v>31</v>
+      </c>
+      <c r="GO5" t="s">
+        <v>17</v>
+      </c>
+      <c r="GP5" t="s">
+        <v>18</v>
+      </c>
+      <c r="GQ5" t="s">
+        <v>19</v>
+      </c>
+      <c r="GR5" t="s">
+        <v>13</v>
+      </c>
+      <c r="GS5" t="s">
+        <v>36</v>
+      </c>
+      <c r="GT5" t="s">
+        <v>6</v>
+      </c>
+      <c r="GU5" t="s">
+        <v>13</v>
+      </c>
+      <c r="GV5" t="s">
+        <v>14</v>
+      </c>
+      <c r="GW5" t="s">
+        <v>27</v>
+      </c>
+      <c r="GX5" t="s">
+        <v>13</v>
+      </c>
+      <c r="GY5" t="s">
+        <v>136</v>
+      </c>
+      <c r="GZ5" t="s">
+        <v>8</v>
+      </c>
+      <c r="HA5" t="s">
+        <v>8</v>
+      </c>
+      <c r="HB5" t="s">
+        <v>0</v>
+      </c>
+      <c r="HC5" t="s">
+        <v>33</v>
+      </c>
+      <c r="HD5" t="s">
+        <v>22</v>
+      </c>
+      <c r="HE5" t="s">
+        <v>31</v>
+      </c>
+      <c r="HF5" t="s">
+        <v>17</v>
+      </c>
+      <c r="HG5" t="s">
+        <v>18</v>
+      </c>
+      <c r="HH5" t="s">
+        <v>19</v>
+      </c>
+      <c r="HI5" t="s">
+        <v>13</v>
+      </c>
+      <c r="HJ5" t="s">
+        <v>38</v>
+      </c>
+      <c r="HK5" t="s">
+        <v>6</v>
+      </c>
+      <c r="HL5" t="s">
+        <v>13</v>
+      </c>
+      <c r="HM5" t="s">
+        <v>14</v>
+      </c>
+      <c r="HN5" t="s">
+        <v>10</v>
+      </c>
+      <c r="HO5" t="s">
+        <v>39</v>
+      </c>
+      <c r="HP5" t="s">
+        <v>137</v>
+      </c>
+      <c r="HQ5" t="s">
+        <v>8</v>
+      </c>
+      <c r="HR5" t="s">
+        <v>8</v>
+      </c>
+      <c r="HS5" t="s">
+        <v>0</v>
+      </c>
+      <c r="HT5" t="s">
+        <v>41</v>
+      </c>
+      <c r="HU5" t="s">
+        <v>22</v>
+      </c>
+      <c r="HV5" t="s">
+        <v>138</v>
+      </c>
+      <c r="HW5" t="s">
+        <v>41</v>
+      </c>
+      <c r="HX5" t="s">
+        <v>139</v>
+      </c>
+      <c r="HY5" t="s">
+        <v>24</v>
+      </c>
+      <c r="HZ5" t="s">
+        <v>140</v>
+      </c>
+      <c r="IA5" t="s">
+        <v>11</v>
+      </c>
+      <c r="IB5" t="s">
+        <v>8</v>
+      </c>
+      <c r="IC5" t="s">
+        <v>104</v>
+      </c>
+      <c r="ID5" t="s">
+        <v>141</v>
+      </c>
+      <c r="IE5" t="s">
+        <v>29</v>
+      </c>
+      <c r="IF5" t="s">
+        <v>34</v>
+      </c>
+      <c r="IG5" t="s">
+        <v>104</v>
+      </c>
+      <c r="IH5" t="s">
+        <v>104</v>
+      </c>
+      <c r="II5" t="s">
+        <v>85</v>
+      </c>
+      <c r="IJ5" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="6" spans="1:258" x14ac:dyDescent="0.25">
+      <c r="A6"/>
+      <c r="B6" t="s">
+        <v>72</v>
+      </c>
+      <c r="C6" t="s">
+        <v>1</v>
+      </c>
+      <c r="D6" t="s">
+        <v>13</v>
+      </c>
+      <c r="E6" t="s">
+        <v>1</v>
+      </c>
+      <c r="F6" t="s">
+        <v>83</v>
+      </c>
+      <c r="G6" t="s">
+        <v>73</v>
+      </c>
+      <c r="H6" t="s">
+        <v>6</v>
+      </c>
+      <c r="I6" t="s">
+        <v>74</v>
+      </c>
+      <c r="J6" t="s">
+        <v>4</v>
+      </c>
+      <c r="K6" t="s">
+        <v>75</v>
+      </c>
+      <c r="L6" t="s">
+        <v>9</v>
+      </c>
+      <c r="M6" t="s">
+        <v>84</v>
+      </c>
+      <c r="N6" t="s">
+        <v>85</v>
+      </c>
+      <c r="O6" t="s">
+        <v>9</v>
+      </c>
+      <c r="P6" t="s">
+        <v>13</v>
+      </c>
+      <c r="Q6" t="s">
+        <v>76</v>
+      </c>
+      <c r="R6" t="s">
+        <v>77</v>
+      </c>
+      <c r="S6" t="s">
+        <v>1</v>
+      </c>
+      <c r="T6" t="s">
+        <v>8</v>
+      </c>
+      <c r="U6" t="s">
+        <v>16</v>
+      </c>
+      <c r="V6" t="s">
+        <v>17</v>
+      </c>
+      <c r="W6" t="s">
+        <v>73</v>
+      </c>
+      <c r="X6" t="s">
+        <v>6</v>
+      </c>
+      <c r="Y6" t="s">
+        <v>74</v>
+      </c>
+      <c r="Z6" t="s">
+        <v>4</v>
+      </c>
+      <c r="AA6" t="s">
+        <v>75</v>
+      </c>
+      <c r="AB6" t="s">
+        <v>9</v>
+      </c>
+      <c r="AC6" t="s">
+        <v>84</v>
+      </c>
+      <c r="AD6" t="s">
+        <v>85</v>
+      </c>
+      <c r="AE6" t="s">
+        <v>9</v>
+      </c>
+      <c r="AF6" t="s">
+        <v>13</v>
+      </c>
+      <c r="AG6" t="s">
+        <v>76</v>
+      </c>
+      <c r="AH6" t="s">
+        <v>77</v>
+      </c>
+      <c r="AI6" t="s">
+        <v>1</v>
+      </c>
+      <c r="AJ6" t="s">
+        <v>17</v>
+      </c>
+      <c r="AK6" t="s">
+        <v>18</v>
+      </c>
+      <c r="AL6" t="s">
+        <v>19</v>
+      </c>
+      <c r="AM6" t="s">
+        <v>13</v>
+      </c>
+      <c r="AN6" t="s">
+        <v>19</v>
+      </c>
+      <c r="AO6" t="s">
+        <v>20</v>
+      </c>
+      <c r="AP6" t="s">
+        <v>13</v>
+      </c>
+      <c r="AQ6" t="s">
+        <v>76</v>
+      </c>
+      <c r="AR6" t="s">
+        <v>18</v>
+      </c>
+      <c r="AS6" t="s">
+        <v>13</v>
+      </c>
+      <c r="AT6" t="s">
+        <v>17</v>
+      </c>
+      <c r="AU6" t="s">
+        <v>86</v>
+      </c>
+      <c r="AV6" t="s">
+        <v>78</v>
+      </c>
+      <c r="AW6" t="s">
+        <v>8</v>
+      </c>
+      <c r="AX6" t="s">
+        <v>8</v>
+      </c>
+      <c r="AY6" t="s">
+        <v>72</v>
+      </c>
+      <c r="AZ6" t="s">
+        <v>13</v>
+      </c>
+      <c r="BA6" t="s">
+        <v>22</v>
+      </c>
+      <c r="BB6" t="s">
+        <v>79</v>
+      </c>
+      <c r="BC6" t="s">
+        <v>17</v>
+      </c>
+      <c r="BD6" t="s">
+        <v>18</v>
+      </c>
+      <c r="BE6" t="s">
+        <v>19</v>
+      </c>
+      <c r="BF6" t="s">
+        <v>13</v>
+      </c>
+      <c r="BG6" t="s">
+        <v>8</v>
+      </c>
+      <c r="BH6" t="s">
+        <v>20</v>
+      </c>
+      <c r="BI6" t="s">
+        <v>13</v>
+      </c>
+      <c r="BJ6" t="s">
+        <v>76</v>
+      </c>
+      <c r="BK6" t="s">
+        <v>18</v>
+      </c>
+      <c r="BL6" t="s">
+        <v>13</v>
+      </c>
+      <c r="BM6" t="s">
+        <v>13</v>
+      </c>
+      <c r="BN6" t="s">
+        <v>13</v>
+      </c>
+      <c r="BO6" t="s">
+        <v>13</v>
+      </c>
+      <c r="BP6" t="s">
+        <v>8</v>
+      </c>
+      <c r="BQ6" t="s">
+        <v>8</v>
+      </c>
+      <c r="BR6" t="s">
+        <v>72</v>
+      </c>
+      <c r="BS6" t="s">
+        <v>13</v>
+      </c>
+      <c r="BT6" t="s">
+        <v>22</v>
+      </c>
+      <c r="BU6" t="s">
+        <v>79</v>
+      </c>
+      <c r="BV6" t="s">
+        <v>17</v>
+      </c>
+      <c r="BW6" t="s">
+        <v>18</v>
+      </c>
+      <c r="BX6" t="s">
+        <v>19</v>
+      </c>
+      <c r="BY6" t="s">
+        <v>13</v>
+      </c>
+      <c r="BZ6" t="s">
+        <v>19</v>
+      </c>
+      <c r="CA6" t="s">
+        <v>6</v>
+      </c>
+      <c r="CB6" t="s">
+        <v>13</v>
+      </c>
+      <c r="CC6" t="s">
+        <v>76</v>
+      </c>
+      <c r="CD6" t="s">
+        <v>18</v>
+      </c>
+      <c r="CE6" t="s">
+        <v>13</v>
+      </c>
+      <c r="CF6" t="s">
+        <v>13</v>
+      </c>
+      <c r="CG6" t="s">
+        <v>8</v>
+      </c>
+      <c r="CH6" t="s">
+        <v>39</v>
+      </c>
+      <c r="CI6" t="s">
+        <v>8</v>
+      </c>
+      <c r="CJ6" t="s">
+        <v>8</v>
+      </c>
+      <c r="CK6" t="s">
+        <v>72</v>
+      </c>
+      <c r="CL6" t="s">
+        <v>13</v>
+      </c>
+      <c r="CM6" t="s">
+        <v>22</v>
+      </c>
+      <c r="CN6" t="s">
+        <v>80</v>
+      </c>
+      <c r="CO6" t="s">
+        <v>17</v>
+      </c>
+      <c r="CP6" t="s">
+        <v>18</v>
+      </c>
+      <c r="CQ6" t="s">
+        <v>19</v>
+      </c>
+      <c r="CR6" t="s">
+        <v>13</v>
+      </c>
+      <c r="CS6" t="s">
+        <v>8</v>
+      </c>
+      <c r="CT6" t="s">
+        <v>6</v>
+      </c>
+      <c r="CU6" t="s">
+        <v>13</v>
+      </c>
+      <c r="CV6" t="s">
+        <v>76</v>
+      </c>
+      <c r="CW6" t="s">
+        <v>18</v>
+      </c>
+      <c r="CX6" t="s">
+        <v>13</v>
+      </c>
+      <c r="CY6" t="s">
+        <v>13</v>
+      </c>
+      <c r="CZ6" t="s">
+        <v>13</v>
+      </c>
+      <c r="DA6" t="s">
+        <v>13</v>
+      </c>
+      <c r="DB6" t="s">
+        <v>8</v>
+      </c>
+      <c r="DC6" t="s">
+        <v>8</v>
+      </c>
+      <c r="DD6" t="s">
+        <v>72</v>
+      </c>
+      <c r="DE6" t="s">
+        <v>13</v>
+      </c>
+      <c r="DF6" t="s">
+        <v>22</v>
+      </c>
+      <c r="DG6" t="s">
+        <v>80</v>
+      </c>
+      <c r="DH6" t="s">
+        <v>17</v>
+      </c>
+      <c r="DI6" t="s">
+        <v>18</v>
+      </c>
+      <c r="DJ6" t="s">
+        <v>19</v>
+      </c>
+      <c r="DK6" t="s">
+        <v>13</v>
+      </c>
+      <c r="DL6" t="s">
+        <v>26</v>
+      </c>
+      <c r="DM6" t="s">
+        <v>6</v>
+      </c>
+      <c r="DN6" t="s">
+        <v>13</v>
+      </c>
+      <c r="DO6" t="s">
+        <v>76</v>
+      </c>
+      <c r="DP6" t="s">
+        <v>27</v>
+      </c>
+      <c r="DQ6" t="s">
+        <v>17</v>
+      </c>
+      <c r="DR6" t="s">
+        <v>87</v>
+      </c>
+      <c r="DS6" t="s">
+        <v>8</v>
+      </c>
+      <c r="DT6" t="s">
+        <v>8</v>
+      </c>
+      <c r="DU6" t="s">
+        <v>72</v>
+      </c>
+      <c r="DV6" t="s">
+        <v>76</v>
+      </c>
+      <c r="DW6" t="s">
+        <v>22</v>
+      </c>
+      <c r="DX6" t="s">
+        <v>16</v>
+      </c>
+      <c r="DY6" t="s">
+        <v>17</v>
+      </c>
+      <c r="DZ6" t="s">
+        <v>18</v>
+      </c>
+      <c r="EA6" t="s">
+        <v>19</v>
+      </c>
+      <c r="EB6" t="s">
+        <v>13</v>
+      </c>
+      <c r="EC6" t="s">
+        <v>29</v>
+      </c>
+      <c r="ED6" t="s">
+        <v>6</v>
+      </c>
+      <c r="EE6" t="s">
+        <v>13</v>
+      </c>
+      <c r="EF6" t="s">
+        <v>76</v>
+      </c>
+      <c r="EG6" t="s">
+        <v>27</v>
+      </c>
+      <c r="EH6" t="s">
+        <v>17</v>
+      </c>
+      <c r="EI6" t="s">
+        <v>88</v>
+      </c>
+      <c r="EJ6" t="s">
+        <v>8</v>
+      </c>
+      <c r="EK6" t="s">
+        <v>8</v>
+      </c>
+      <c r="EL6" t="s">
+        <v>72</v>
+      </c>
+      <c r="EM6" t="s">
+        <v>76</v>
+      </c>
+      <c r="EN6" t="s">
+        <v>22</v>
+      </c>
+      <c r="EO6" t="s">
+        <v>16</v>
+      </c>
+      <c r="EP6" t="s">
+        <v>17</v>
+      </c>
+      <c r="EQ6" t="s">
+        <v>18</v>
+      </c>
+      <c r="ER6" t="s">
+        <v>19</v>
+      </c>
+      <c r="ES6" t="s">
+        <v>13</v>
+      </c>
+      <c r="ET6" t="s">
+        <v>30</v>
+      </c>
+      <c r="EU6" t="s">
+        <v>6</v>
+      </c>
+      <c r="EV6" t="s">
+        <v>13</v>
+      </c>
+      <c r="EW6" t="s">
+        <v>76</v>
+      </c>
+      <c r="EX6" t="s">
+        <v>27</v>
+      </c>
+      <c r="EY6" t="s">
+        <v>17</v>
+      </c>
+      <c r="EZ6" t="s">
+        <v>89</v>
+      </c>
+      <c r="FA6" t="s">
+        <v>8</v>
+      </c>
+      <c r="FB6" t="s">
+        <v>8</v>
+      </c>
+      <c r="FC6" t="s">
+        <v>72</v>
+      </c>
+      <c r="FD6" t="s">
+        <v>76</v>
+      </c>
+      <c r="FE6" t="s">
+        <v>22</v>
+      </c>
+      <c r="FF6" t="s">
+        <v>16</v>
+      </c>
+      <c r="FG6" t="s">
+        <v>17</v>
+      </c>
+      <c r="FH6" t="s">
+        <v>18</v>
+      </c>
+      <c r="FI6" t="s">
+        <v>19</v>
+      </c>
+      <c r="FJ6" t="s">
+        <v>13</v>
+      </c>
+      <c r="FK6" t="s">
+        <v>81</v>
+      </c>
+      <c r="FL6" t="s">
+        <v>6</v>
+      </c>
+      <c r="FM6" t="s">
+        <v>13</v>
+      </c>
+      <c r="FN6" t="s">
+        <v>76</v>
+      </c>
+      <c r="FO6" t="s">
+        <v>27</v>
+      </c>
+      <c r="FP6" t="s">
+        <v>13</v>
+      </c>
+      <c r="FQ6" t="s">
+        <v>90</v>
+      </c>
+      <c r="FR6" t="s">
+        <v>8</v>
+      </c>
+      <c r="FS6" t="s">
+        <v>8</v>
+      </c>
+      <c r="FT6" t="s">
+        <v>72</v>
+      </c>
+      <c r="FU6" t="s">
+        <v>82</v>
+      </c>
+      <c r="FV6" t="s">
+        <v>22</v>
+      </c>
+      <c r="FW6" t="s">
+        <v>31</v>
+      </c>
+      <c r="FX6" t="s">
+        <v>17</v>
+      </c>
+      <c r="FY6" t="s">
+        <v>18</v>
+      </c>
+      <c r="FZ6" t="s">
+        <v>19</v>
+      </c>
+      <c r="GA6" t="s">
+        <v>13</v>
+      </c>
+      <c r="GB6" t="s">
+        <v>34</v>
+      </c>
+      <c r="GC6" t="s">
+        <v>6</v>
+      </c>
+      <c r="GD6" t="s">
+        <v>13</v>
+      </c>
+      <c r="GE6" t="s">
+        <v>76</v>
+      </c>
+      <c r="GF6" t="s">
+        <v>27</v>
+      </c>
+      <c r="GG6" t="s">
+        <v>13</v>
+      </c>
+      <c r="GH6" t="s">
+        <v>91</v>
+      </c>
+      <c r="GI6" t="s">
+        <v>8</v>
+      </c>
+      <c r="GJ6" t="s">
+        <v>8</v>
+      </c>
+      <c r="GK6" t="s">
+        <v>72</v>
+      </c>
+      <c r="GL6" t="s">
+        <v>82</v>
+      </c>
+      <c r="GM6" t="s">
+        <v>22</v>
+      </c>
+      <c r="GN6" t="s">
+        <v>31</v>
+      </c>
+      <c r="GO6" t="s">
+        <v>17</v>
+      </c>
+      <c r="GP6" t="s">
+        <v>18</v>
+      </c>
+      <c r="GQ6" t="s">
+        <v>19</v>
+      </c>
+      <c r="GR6" t="s">
+        <v>13</v>
+      </c>
+      <c r="GS6" t="s">
+        <v>36</v>
+      </c>
+      <c r="GT6" t="s">
+        <v>6</v>
+      </c>
+      <c r="GU6" t="s">
+        <v>13</v>
+      </c>
+      <c r="GV6" t="s">
+        <v>76</v>
+      </c>
+      <c r="GW6" t="s">
+        <v>27</v>
+      </c>
+      <c r="GX6" t="s">
+        <v>13</v>
+      </c>
+      <c r="GY6" t="s">
+        <v>101</v>
+      </c>
+      <c r="GZ6" t="s">
+        <v>8</v>
+      </c>
+      <c r="HA6" t="s">
+        <v>8</v>
+      </c>
+      <c r="HB6" t="s">
+        <v>72</v>
+      </c>
+      <c r="HC6" t="s">
+        <v>82</v>
+      </c>
+      <c r="HD6" t="s">
+        <v>22</v>
+      </c>
+      <c r="HE6" t="s">
+        <v>31</v>
+      </c>
+      <c r="HF6" t="s">
+        <v>17</v>
+      </c>
+      <c r="HG6" t="s">
+        <v>18</v>
+      </c>
+      <c r="HH6" t="s">
+        <v>19</v>
+      </c>
+      <c r="HI6" t="s">
+        <v>13</v>
+      </c>
+      <c r="HJ6" t="s">
+        <v>102</v>
+      </c>
+      <c r="HK6" t="s">
+        <v>6</v>
+      </c>
+      <c r="HL6" t="s">
+        <v>13</v>
+      </c>
+      <c r="HM6" t="s">
+        <v>76</v>
+      </c>
+      <c r="HN6" t="s">
+        <v>10</v>
+      </c>
+      <c r="HO6" t="s">
+        <v>39</v>
+      </c>
+      <c r="HP6" t="s">
+        <v>34</v>
+      </c>
+      <c r="HQ6" t="s">
+        <v>8</v>
+      </c>
+      <c r="HR6" t="s">
+        <v>8</v>
+      </c>
+      <c r="HS6" t="s">
+        <v>72</v>
+      </c>
+      <c r="HT6" t="s">
+        <v>103</v>
+      </c>
+      <c r="HU6" t="s">
+        <v>22</v>
+      </c>
+      <c r="HV6" t="s">
+        <v>76</v>
+      </c>
+      <c r="HW6" t="s">
+        <v>17</v>
+      </c>
+      <c r="HX6" t="s">
+        <v>73</v>
+      </c>
+      <c r="HY6" t="s">
+        <v>104</v>
+      </c>
+      <c r="HZ6" t="s">
+        <v>42</v>
+      </c>
+      <c r="IA6" t="s">
+        <v>85</v>
+      </c>
+      <c r="IB6" t="s">
+        <v>105</v>
+      </c>
+      <c r="IC6" t="s">
+        <v>106</v>
+      </c>
+      <c r="ID6" t="s">
+        <v>107</v>
+      </c>
+      <c r="IE6" t="s">
+        <v>108</v>
+      </c>
+      <c r="IF6" t="s">
+        <v>109</v>
+      </c>
+      <c r="IG6" t="s">
+        <v>110</v>
+      </c>
+      <c r="IH6" t="s">
+        <v>77</v>
+      </c>
+      <c r="II6" t="s">
+        <v>111</v>
+      </c>
+      <c r="IJ6" t="s">
+        <v>112</v>
+      </c>
+      <c r="IK6" t="s">
+        <v>113</v>
+      </c>
+      <c r="IL6" t="s">
+        <v>114</v>
+      </c>
+      <c r="IM6" t="s">
+        <v>115</v>
+      </c>
+      <c r="IN6" t="s">
+        <v>20</v>
+      </c>
+      <c r="IO6" t="s">
+        <v>86</v>
+      </c>
+      <c r="IP6" t="s">
+        <v>87</v>
+      </c>
+      <c r="IQ6" t="s">
+        <v>116</v>
+      </c>
+      <c r="IR6" t="s">
+        <v>117</v>
+      </c>
+      <c r="IS6" t="s">
+        <v>118</v>
+      </c>
+      <c r="IT6" t="s">
+        <v>119</v>
+      </c>
+      <c r="IU6" t="s">
+        <v>120</v>
+      </c>
+      <c r="IV6" t="s">
+        <v>121</v>
+      </c>
+      <c r="IW6" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="7" spans="1:258" s="1" customFormat="1" ht="12" x14ac:dyDescent="0.2">
+      <c r="A7" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="B3" s="1">
+      <c r="B7" s="1">
         <v>0</v>
       </c>
-      <c r="C3" s="1">
-        <f>B3+1</f>
+      <c r="C7" s="1">
+        <f>B7+1</f>
         <v>1</v>
       </c>
-      <c r="D3" s="1">
-        <f t="shared" ref="D3:BO3" si="0">C3+1</f>
+      <c r="D7" s="1">
+        <f t="shared" ref="D7:BO7" si="0">C7+1</f>
         <v>2</v>
       </c>
-      <c r="E3" s="1">
+      <c r="E7" s="1">
         <f t="shared" si="0"/>
         <v>3</v>
       </c>
-      <c r="F3" s="1">
+      <c r="F7" s="1">
         <f t="shared" si="0"/>
         <v>4</v>
       </c>
-      <c r="G3" s="1">
+      <c r="G7" s="1">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="H3" s="1">
+      <c r="H7" s="1">
         <f t="shared" si="0"/>
         <v>6</v>
       </c>
-      <c r="I3" s="1">
+      <c r="I7" s="1">
         <f t="shared" si="0"/>
         <v>7</v>
       </c>
-      <c r="J3" s="1">
-        <f t="shared" si="0"/>
-        <v>8</v>
-      </c>
-      <c r="K3" s="1">
+      <c r="J7" s="1">
+        <f t="shared" si="0"/>
+        <v>8</v>
+      </c>
+      <c r="K7" s="1">
         <f t="shared" si="0"/>
         <v>9</v>
       </c>
-      <c r="L3" s="1">
+      <c r="L7" s="1">
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
-      <c r="M3" s="1">
+      <c r="M7" s="1">
         <f t="shared" si="0"/>
         <v>11</v>
       </c>
-      <c r="N3" s="1">
+      <c r="N7" s="1">
         <f t="shared" si="0"/>
         <v>12</v>
       </c>
-      <c r="O3" s="1">
-        <f t="shared" si="0"/>
-        <v>13</v>
-      </c>
-      <c r="P3" s="1">
+      <c r="O7" s="1">
+        <f t="shared" si="0"/>
+        <v>13</v>
+      </c>
+      <c r="P7" s="1">
         <f t="shared" si="0"/>
         <v>14</v>
       </c>
-      <c r="Q3" s="1">
+      <c r="Q7" s="1">
         <f t="shared" si="0"/>
         <v>15</v>
       </c>
-      <c r="R3" s="1">
+      <c r="R7" s="1">
         <f t="shared" si="0"/>
         <v>16</v>
       </c>
-      <c r="S3" s="1">
+      <c r="S7" s="1">
         <f t="shared" si="0"/>
         <v>17</v>
       </c>
-      <c r="T3" s="1">
+      <c r="T7" s="1">
         <f t="shared" si="0"/>
         <v>18</v>
       </c>
-      <c r="U3" s="1">
+      <c r="U7" s="1">
         <f t="shared" si="0"/>
         <v>19</v>
       </c>
-      <c r="V3" s="1">
+      <c r="V7" s="1">
         <f t="shared" si="0"/>
         <v>20</v>
       </c>
-      <c r="W3" s="1">
+      <c r="W7" s="1">
         <f t="shared" si="0"/>
         <v>21</v>
       </c>
-      <c r="X3" s="1">
+      <c r="X7" s="1">
         <f t="shared" si="0"/>
         <v>22</v>
       </c>
-      <c r="Y3" s="1">
+      <c r="Y7" s="1">
         <f t="shared" si="0"/>
         <v>23</v>
       </c>
-      <c r="Z3" s="1">
+      <c r="Z7" s="1">
         <f t="shared" si="0"/>
         <v>24</v>
       </c>
-      <c r="AA3" s="1">
+      <c r="AA7" s="1">
         <f t="shared" si="0"/>
         <v>25</v>
       </c>
-      <c r="AB3" s="1">
+      <c r="AB7" s="1">
         <f t="shared" si="0"/>
         <v>26</v>
       </c>
-      <c r="AC3" s="1">
+      <c r="AC7" s="1">
         <f t="shared" si="0"/>
         <v>27</v>
       </c>
-      <c r="AD3" s="1">
+      <c r="AD7" s="1">
         <f t="shared" si="0"/>
         <v>28</v>
       </c>
-      <c r="AE3" s="1">
+      <c r="AE7" s="1">
         <f t="shared" si="0"/>
         <v>29</v>
       </c>
-      <c r="AF3" s="1">
+      <c r="AF7" s="1">
         <f t="shared" si="0"/>
         <v>30</v>
       </c>
-      <c r="AG3" s="1">
+      <c r="AG7" s="1">
         <f t="shared" si="0"/>
         <v>31</v>
       </c>
-      <c r="AH3" s="1">
+      <c r="AH7" s="1">
         <f t="shared" si="0"/>
         <v>32</v>
       </c>
-      <c r="AI3" s="1">
+      <c r="AI7" s="1">
         <f t="shared" si="0"/>
         <v>33</v>
       </c>
-      <c r="AJ3" s="1">
+      <c r="AJ7" s="1">
         <f t="shared" si="0"/>
         <v>34</v>
       </c>
-      <c r="AK3" s="1">
+      <c r="AK7" s="1">
         <f t="shared" si="0"/>
         <v>35</v>
       </c>
-      <c r="AL3" s="1">
+      <c r="AL7" s="1">
         <f t="shared" si="0"/>
         <v>36</v>
       </c>
-      <c r="AM3" s="1">
+      <c r="AM7" s="1">
         <f t="shared" si="0"/>
         <v>37</v>
       </c>
-      <c r="AN3" s="1">
+      <c r="AN7" s="1">
         <f t="shared" si="0"/>
         <v>38</v>
       </c>
-      <c r="AO3" s="1">
+      <c r="AO7" s="1">
         <f t="shared" si="0"/>
         <v>39</v>
       </c>
-      <c r="AP3" s="1">
+      <c r="AP7" s="1">
         <f t="shared" si="0"/>
         <v>40</v>
       </c>
-      <c r="AQ3" s="1">
+      <c r="AQ7" s="1">
         <f t="shared" si="0"/>
         <v>41</v>
       </c>
-      <c r="AR3" s="1">
+      <c r="AR7" s="1">
         <f t="shared" si="0"/>
         <v>42</v>
       </c>
-      <c r="AS3" s="1">
+      <c r="AS7" s="1">
         <f t="shared" si="0"/>
         <v>43</v>
       </c>
-      <c r="AT3" s="1">
+      <c r="AT7" s="1">
         <f t="shared" si="0"/>
         <v>44</v>
       </c>
-      <c r="AU3" s="1">
+      <c r="AU7" s="1">
         <f t="shared" si="0"/>
         <v>45</v>
       </c>
-      <c r="AV3" s="1">
+      <c r="AV7" s="1">
         <f t="shared" si="0"/>
         <v>46</v>
       </c>
-      <c r="AW3" s="1">
+      <c r="AW7" s="1">
         <f t="shared" si="0"/>
         <v>47</v>
       </c>
-      <c r="AX3" s="1">
+      <c r="AX7" s="1">
         <f t="shared" si="0"/>
         <v>48</v>
       </c>
-      <c r="AY3" s="1">
+      <c r="AY7" s="1">
         <f t="shared" si="0"/>
         <v>49</v>
       </c>
-      <c r="AZ3" s="1">
+      <c r="AZ7" s="1">
         <f t="shared" si="0"/>
         <v>50</v>
       </c>
-      <c r="BA3" s="1">
+      <c r="BA7" s="1">
         <f t="shared" si="0"/>
         <v>51</v>
       </c>
-      <c r="BB3" s="1">
+      <c r="BB7" s="1">
         <f t="shared" si="0"/>
         <v>52</v>
       </c>
-      <c r="BC3" s="1">
+      <c r="BC7" s="1">
         <f t="shared" si="0"/>
         <v>53</v>
       </c>
-      <c r="BD3" s="1">
+      <c r="BD7" s="1">
         <f t="shared" si="0"/>
         <v>54</v>
       </c>
-      <c r="BE3" s="1">
+      <c r="BE7" s="1">
         <f t="shared" si="0"/>
         <v>55</v>
       </c>
-      <c r="BF3" s="1">
+      <c r="BF7" s="1">
         <f t="shared" si="0"/>
         <v>56</v>
       </c>
-      <c r="BG3" s="1">
+      <c r="BG7" s="1">
         <f t="shared" si="0"/>
         <v>57</v>
       </c>
-      <c r="BH3" s="1">
+      <c r="BH7" s="1">
         <f t="shared" si="0"/>
         <v>58</v>
       </c>
-      <c r="BI3" s="1">
+      <c r="BI7" s="1">
         <f t="shared" si="0"/>
         <v>59</v>
       </c>
-      <c r="BJ3" s="1">
+      <c r="BJ7" s="1">
         <f t="shared" si="0"/>
         <v>60</v>
       </c>
-      <c r="BK3" s="1">
+      <c r="BK7" s="1">
         <f t="shared" si="0"/>
         <v>61</v>
       </c>
-      <c r="BL3" s="1">
+      <c r="BL7" s="1">
         <f t="shared" si="0"/>
         <v>62</v>
       </c>
-      <c r="BM3" s="1">
+      <c r="BM7" s="1">
         <f t="shared" si="0"/>
         <v>63</v>
       </c>
-      <c r="BN3" s="1">
+      <c r="BN7" s="1">
         <f t="shared" si="0"/>
         <v>64</v>
       </c>
-      <c r="BO3" s="1">
+      <c r="BO7" s="1">
         <f t="shared" si="0"/>
         <v>65</v>
       </c>
-      <c r="BP3" s="1">
-        <f t="shared" ref="BP3:EA3" si="1">BO3+1</f>
+      <c r="BP7" s="1">
+        <f t="shared" ref="BP7:EA7" si="1">BO7+1</f>
         <v>66</v>
       </c>
-      <c r="BQ3" s="1">
+      <c r="BQ7" s="1">
         <f t="shared" si="1"/>
         <v>67</v>
       </c>
-      <c r="BR3" s="1">
+      <c r="BR7" s="1">
         <f t="shared" si="1"/>
         <v>68</v>
       </c>
-      <c r="BS3" s="1">
+      <c r="BS7" s="1">
         <f t="shared" si="1"/>
         <v>69</v>
       </c>
-      <c r="BT3" s="1">
+      <c r="BT7" s="1">
         <f t="shared" si="1"/>
         <v>70</v>
       </c>
-      <c r="BU3" s="1">
+      <c r="BU7" s="1">
         <f t="shared" si="1"/>
         <v>71</v>
       </c>
-      <c r="BV3" s="1">
+      <c r="BV7" s="1">
         <f t="shared" si="1"/>
         <v>72</v>
       </c>
-      <c r="BW3" s="1">
+      <c r="BW7" s="1">
         <f t="shared" si="1"/>
         <v>73</v>
       </c>
-      <c r="BX3" s="1">
+      <c r="BX7" s="1">
         <f t="shared" si="1"/>
         <v>74</v>
       </c>
-      <c r="BY3" s="1">
+      <c r="BY7" s="1">
         <f t="shared" si="1"/>
         <v>75</v>
       </c>
-      <c r="BZ3" s="1">
+      <c r="BZ7" s="1">
         <f t="shared" si="1"/>
         <v>76</v>
       </c>
-      <c r="CA3" s="1">
+      <c r="CA7" s="1">
         <f t="shared" si="1"/>
         <v>77</v>
       </c>
-      <c r="CB3" s="1">
+      <c r="CB7" s="1">
         <f t="shared" si="1"/>
         <v>78</v>
       </c>
-      <c r="CC3" s="1">
+      <c r="CC7" s="1">
         <f t="shared" si="1"/>
         <v>79</v>
       </c>
-      <c r="CD3" s="1">
+      <c r="CD7" s="1">
         <f t="shared" si="1"/>
         <v>80</v>
       </c>
-      <c r="CE3" s="1">
+      <c r="CE7" s="1">
         <f t="shared" si="1"/>
         <v>81</v>
       </c>
-      <c r="CF3" s="1">
+      <c r="CF7" s="1">
         <f t="shared" si="1"/>
         <v>82</v>
       </c>
-      <c r="CG3" s="1">
+      <c r="CG7" s="1">
         <f t="shared" si="1"/>
         <v>83</v>
       </c>
-      <c r="CH3" s="1">
+      <c r="CH7" s="1">
         <f t="shared" si="1"/>
         <v>84</v>
       </c>
-      <c r="CI3" s="1">
+      <c r="CI7" s="1">
         <f t="shared" si="1"/>
         <v>85</v>
       </c>
-      <c r="CJ3" s="1">
+      <c r="CJ7" s="1">
         <f t="shared" si="1"/>
         <v>86</v>
       </c>
-      <c r="CK3" s="1">
+      <c r="CK7" s="1">
         <f t="shared" si="1"/>
         <v>87</v>
       </c>
-      <c r="CL3" s="1">
+      <c r="CL7" s="1">
         <f t="shared" si="1"/>
         <v>88</v>
       </c>
-      <c r="CM3" s="1">
+      <c r="CM7" s="1">
         <f t="shared" si="1"/>
         <v>89</v>
       </c>
-      <c r="CN3" s="1">
+      <c r="CN7" s="1">
         <f t="shared" si="1"/>
         <v>90</v>
       </c>
-      <c r="CO3" s="1">
+      <c r="CO7" s="1">
         <f t="shared" si="1"/>
         <v>91</v>
       </c>
-      <c r="CP3" s="1">
+      <c r="CP7" s="1">
         <f t="shared" si="1"/>
         <v>92</v>
       </c>
-      <c r="CQ3" s="1">
+      <c r="CQ7" s="1">
         <f t="shared" si="1"/>
         <v>93</v>
       </c>
-      <c r="CR3" s="1">
+      <c r="CR7" s="1">
         <f t="shared" si="1"/>
         <v>94</v>
       </c>
-      <c r="CS3" s="1">
+      <c r="CS7" s="1">
         <f t="shared" si="1"/>
         <v>95</v>
       </c>
-      <c r="CT3" s="1">
+      <c r="CT7" s="1">
         <f t="shared" si="1"/>
         <v>96</v>
       </c>
-      <c r="CU3" s="1">
+      <c r="CU7" s="1">
         <f t="shared" si="1"/>
         <v>97</v>
       </c>
-      <c r="CV3" s="1">
+      <c r="CV7" s="1">
         <f t="shared" si="1"/>
         <v>98</v>
       </c>
-      <c r="CW3" s="1">
+      <c r="CW7" s="1">
         <f t="shared" si="1"/>
         <v>99</v>
       </c>
-      <c r="CX3" s="1">
+      <c r="CX7" s="1">
         <f t="shared" si="1"/>
         <v>100</v>
       </c>
-      <c r="CY3" s="1">
+      <c r="CY7" s="1">
         <f t="shared" si="1"/>
         <v>101</v>
       </c>
-      <c r="CZ3" s="1">
+      <c r="CZ7" s="1">
         <f t="shared" si="1"/>
         <v>102</v>
       </c>
-      <c r="DA3" s="1">
+      <c r="DA7" s="1">
         <f t="shared" si="1"/>
         <v>103</v>
       </c>
-      <c r="DB3" s="1">
+      <c r="DB7" s="1">
         <f t="shared" si="1"/>
         <v>104</v>
       </c>
-      <c r="DC3" s="1">
+      <c r="DC7" s="1">
         <f t="shared" si="1"/>
         <v>105</v>
       </c>
-      <c r="DD3" s="1">
+      <c r="DD7" s="1">
         <f t="shared" si="1"/>
         <v>106</v>
       </c>
-      <c r="DE3" s="1">
+      <c r="DE7" s="1">
         <f t="shared" si="1"/>
         <v>107</v>
       </c>
-      <c r="DF3" s="1">
+      <c r="DF7" s="1">
         <f t="shared" si="1"/>
         <v>108</v>
       </c>
-      <c r="DG3" s="1">
+      <c r="DG7" s="1">
         <f t="shared" si="1"/>
         <v>109</v>
       </c>
-      <c r="DH3" s="1">
+      <c r="DH7" s="1">
         <f t="shared" si="1"/>
         <v>110</v>
       </c>
-      <c r="DI3" s="1">
+      <c r="DI7" s="1">
         <f t="shared" si="1"/>
         <v>111</v>
       </c>
-      <c r="DJ3" s="1">
+      <c r="DJ7" s="1">
         <f t="shared" si="1"/>
         <v>112</v>
       </c>
-      <c r="DK3" s="1">
+      <c r="DK7" s="1">
         <f t="shared" si="1"/>
         <v>113</v>
       </c>
-      <c r="DL3" s="1">
+      <c r="DL7" s="1">
         <f t="shared" si="1"/>
         <v>114</v>
       </c>
-      <c r="DM3" s="1">
+      <c r="DM7" s="1">
         <f t="shared" si="1"/>
         <v>115</v>
       </c>
-      <c r="DN3" s="1">
+      <c r="DN7" s="1">
         <f t="shared" si="1"/>
         <v>116</v>
       </c>
-      <c r="DO3" s="1">
+      <c r="DO7" s="1">
         <f t="shared" si="1"/>
         <v>117</v>
       </c>
-      <c r="DP3" s="1">
+      <c r="DP7" s="1">
         <f t="shared" si="1"/>
         <v>118</v>
       </c>
-      <c r="DQ3" s="1">
+      <c r="DQ7" s="1">
         <f t="shared" si="1"/>
         <v>119</v>
       </c>
-      <c r="DR3" s="1">
+      <c r="DR7" s="1">
         <f t="shared" si="1"/>
         <v>120</v>
       </c>
-      <c r="DS3" s="1">
+      <c r="DS7" s="1">
         <f t="shared" si="1"/>
         <v>121</v>
       </c>
-      <c r="DT3" s="1">
+      <c r="DT7" s="1">
         <f t="shared" si="1"/>
         <v>122</v>
       </c>
-      <c r="DU3" s="1">
+      <c r="DU7" s="1">
         <f t="shared" si="1"/>
         <v>123</v>
       </c>
-      <c r="DV3" s="1">
+      <c r="DV7" s="1">
         <f t="shared" si="1"/>
         <v>124</v>
       </c>
-      <c r="DW3" s="1">
+      <c r="DW7" s="1">
         <f t="shared" si="1"/>
         <v>125</v>
       </c>
-      <c r="DX3" s="1">
+      <c r="DX7" s="1">
         <f t="shared" si="1"/>
         <v>126</v>
       </c>
-      <c r="DY3" s="1">
+      <c r="DY7" s="1">
         <f t="shared" si="1"/>
         <v>127</v>
       </c>
-      <c r="DZ3" s="1">
+      <c r="DZ7" s="1">
         <f t="shared" si="1"/>
         <v>128</v>
       </c>
-      <c r="EA3" s="1">
+      <c r="EA7" s="1">
         <f t="shared" si="1"/>
         <v>129</v>
       </c>
-      <c r="EB3" s="1">
-        <f t="shared" ref="EB3:GM3" si="2">EA3+1</f>
+      <c r="EB7" s="1">
+        <f t="shared" ref="EB7:GM7" si="2">EA7+1</f>
         <v>130</v>
       </c>
-      <c r="EC3" s="1">
+      <c r="EC7" s="1">
         <f t="shared" si="2"/>
         <v>131</v>
       </c>
-      <c r="ED3" s="1">
+      <c r="ED7" s="1">
         <f t="shared" si="2"/>
         <v>132</v>
       </c>
-      <c r="EE3" s="1">
+      <c r="EE7" s="1">
         <f t="shared" si="2"/>
         <v>133</v>
       </c>
-      <c r="EF3" s="1">
+      <c r="EF7" s="1">
         <f t="shared" si="2"/>
         <v>134</v>
       </c>
-      <c r="EG3" s="1">
+      <c r="EG7" s="1">
         <f t="shared" si="2"/>
         <v>135</v>
       </c>
-      <c r="EH3" s="1">
+      <c r="EH7" s="1">
         <f t="shared" si="2"/>
         <v>136</v>
       </c>
-      <c r="EI3" s="1">
+      <c r="EI7" s="1">
         <f t="shared" si="2"/>
         <v>137</v>
       </c>
-      <c r="EJ3" s="1">
+      <c r="EJ7" s="1">
         <f t="shared" si="2"/>
         <v>138</v>
       </c>
-      <c r="EK3" s="1">
+      <c r="EK7" s="1">
         <f t="shared" si="2"/>
         <v>139</v>
       </c>
-      <c r="EL3" s="1">
+      <c r="EL7" s="1">
         <f t="shared" si="2"/>
         <v>140</v>
       </c>
-      <c r="EM3" s="1">
+      <c r="EM7" s="1">
         <f t="shared" si="2"/>
         <v>141</v>
       </c>
-      <c r="EN3" s="1">
+      <c r="EN7" s="1">
         <f t="shared" si="2"/>
         <v>142</v>
       </c>
-      <c r="EO3" s="1">
+      <c r="EO7" s="1">
         <f t="shared" si="2"/>
         <v>143</v>
       </c>
-      <c r="EP3" s="1">
+      <c r="EP7" s="1">
         <f t="shared" si="2"/>
         <v>144</v>
       </c>
-      <c r="EQ3" s="1">
+      <c r="EQ7" s="1">
         <f t="shared" si="2"/>
         <v>145</v>
       </c>
-      <c r="ER3" s="1">
+      <c r="ER7" s="1">
         <f t="shared" si="2"/>
         <v>146</v>
       </c>
-      <c r="ES3" s="1">
+      <c r="ES7" s="1">
         <f t="shared" si="2"/>
         <v>147</v>
       </c>
-      <c r="ET3" s="1">
+      <c r="ET7" s="1">
         <f t="shared" si="2"/>
         <v>148</v>
       </c>
-      <c r="EU3" s="1">
+      <c r="EU7" s="1">
         <f t="shared" si="2"/>
         <v>149</v>
       </c>
-      <c r="EV3" s="1">
+      <c r="EV7" s="1">
         <f t="shared" si="2"/>
         <v>150</v>
       </c>
-      <c r="EW3" s="1">
+      <c r="EW7" s="1">
         <f t="shared" si="2"/>
         <v>151</v>
       </c>
-      <c r="EX3" s="1">
+      <c r="EX7" s="1">
         <f t="shared" si="2"/>
         <v>152</v>
       </c>
-      <c r="EY3" s="1">
+      <c r="EY7" s="1">
         <f t="shared" si="2"/>
         <v>153</v>
       </c>
-      <c r="EZ3" s="1">
+      <c r="EZ7" s="1">
         <f t="shared" si="2"/>
         <v>154</v>
       </c>
-      <c r="FA3" s="1">
+      <c r="FA7" s="1">
         <f t="shared" si="2"/>
         <v>155</v>
       </c>
-      <c r="FB3" s="1">
+      <c r="FB7" s="1">
         <f t="shared" si="2"/>
         <v>156</v>
       </c>
-      <c r="FC3" s="1">
+      <c r="FC7" s="1">
         <f t="shared" si="2"/>
         <v>157</v>
       </c>
-      <c r="FD3" s="1">
+      <c r="FD7" s="1">
         <f t="shared" si="2"/>
         <v>158</v>
       </c>
-      <c r="FE3" s="1">
+      <c r="FE7" s="1">
         <f t="shared" si="2"/>
         <v>159</v>
       </c>
-      <c r="FF3" s="1">
+      <c r="FF7" s="1">
         <f t="shared" si="2"/>
         <v>160</v>
       </c>
-      <c r="FG3" s="1">
+      <c r="FG7" s="1">
         <f t="shared" si="2"/>
         <v>161</v>
       </c>
-      <c r="FH3" s="1">
+      <c r="FH7" s="1">
         <f t="shared" si="2"/>
         <v>162</v>
       </c>
-      <c r="FI3" s="1">
+      <c r="FI7" s="1">
         <f t="shared" si="2"/>
         <v>163</v>
       </c>
-      <c r="FJ3" s="1">
+      <c r="FJ7" s="1">
         <f t="shared" si="2"/>
         <v>164</v>
       </c>
-      <c r="FK3" s="1">
+      <c r="FK7" s="1">
         <f t="shared" si="2"/>
         <v>165</v>
       </c>
-      <c r="FL3" s="1">
+      <c r="FL7" s="1">
         <f t="shared" si="2"/>
         <v>166</v>
       </c>
-      <c r="FM3" s="1">
+      <c r="FM7" s="1">
         <f t="shared" si="2"/>
         <v>167</v>
       </c>
-      <c r="FN3" s="1">
+      <c r="FN7" s="1">
         <f t="shared" si="2"/>
         <v>168</v>
       </c>
-      <c r="FO3" s="1">
+      <c r="FO7" s="1">
         <f t="shared" si="2"/>
         <v>169</v>
       </c>
-      <c r="FP3" s="1">
+      <c r="FP7" s="1">
         <f t="shared" si="2"/>
         <v>170</v>
       </c>
-      <c r="FQ3" s="1">
+      <c r="FQ7" s="1">
         <f t="shared" si="2"/>
         <v>171</v>
       </c>
-      <c r="FR3" s="1">
+      <c r="FR7" s="1">
         <f t="shared" si="2"/>
         <v>172</v>
       </c>
-      <c r="FS3" s="1">
+      <c r="FS7" s="1">
         <f t="shared" si="2"/>
         <v>173</v>
       </c>
-      <c r="FT3" s="1">
+      <c r="FT7" s="1">
         <f t="shared" si="2"/>
         <v>174</v>
       </c>
-      <c r="FU3" s="1">
+      <c r="FU7" s="1">
         <f t="shared" si="2"/>
         <v>175</v>
       </c>
-      <c r="FV3" s="1">
+      <c r="FV7" s="1">
         <f t="shared" si="2"/>
         <v>176</v>
       </c>
-      <c r="FW3" s="1">
+      <c r="FW7" s="1">
         <f t="shared" si="2"/>
         <v>177</v>
       </c>
-      <c r="FX3" s="1">
+      <c r="FX7" s="1">
         <f t="shared" si="2"/>
         <v>178</v>
       </c>
-      <c r="FY3" s="1">
+      <c r="FY7" s="1">
         <f t="shared" si="2"/>
         <v>179</v>
       </c>
-      <c r="FZ3" s="1">
+      <c r="FZ7" s="1">
         <f t="shared" si="2"/>
         <v>180</v>
       </c>
-      <c r="GA3" s="1">
+      <c r="GA7" s="1">
         <f t="shared" si="2"/>
         <v>181</v>
       </c>
-      <c r="GB3" s="1">
+      <c r="GB7" s="1">
         <f t="shared" si="2"/>
         <v>182</v>
       </c>
-      <c r="GC3" s="1">
+      <c r="GC7" s="1">
         <f t="shared" si="2"/>
         <v>183</v>
       </c>
-      <c r="GD3" s="1">
+      <c r="GD7" s="1">
         <f t="shared" si="2"/>
         <v>184</v>
       </c>
-      <c r="GE3" s="1">
+      <c r="GE7" s="1">
         <f t="shared" si="2"/>
         <v>185</v>
       </c>
-      <c r="GF3" s="1">
+      <c r="GF7" s="1">
         <f t="shared" si="2"/>
         <v>186</v>
       </c>
-      <c r="GG3" s="1">
+      <c r="GG7" s="1">
         <f t="shared" si="2"/>
         <v>187</v>
       </c>
-      <c r="GH3" s="1">
+      <c r="GH7" s="1">
         <f t="shared" si="2"/>
         <v>188</v>
       </c>
-      <c r="GI3" s="1">
+      <c r="GI7" s="1">
         <f t="shared" si="2"/>
         <v>189</v>
       </c>
-      <c r="GJ3" s="1">
+      <c r="GJ7" s="1">
         <f t="shared" si="2"/>
         <v>190</v>
       </c>
-      <c r="GK3" s="1">
+      <c r="GK7" s="1">
         <f t="shared" si="2"/>
         <v>191</v>
       </c>
-      <c r="GL3" s="1">
+      <c r="GL7" s="1">
         <f t="shared" si="2"/>
         <v>192</v>
       </c>
-      <c r="GM3" s="1">
+      <c r="GM7" s="1">
         <f t="shared" si="2"/>
         <v>193</v>
       </c>
-      <c r="GN3" s="1">
-        <f t="shared" ref="GN3:IJ3" si="3">GM3+1</f>
+      <c r="GN7" s="1">
+        <f t="shared" ref="GN7:IJ7" si="3">GM7+1</f>
         <v>194</v>
       </c>
-      <c r="GO3" s="1">
+      <c r="GO7" s="1">
         <f t="shared" si="3"/>
         <v>195</v>
       </c>
-      <c r="GP3" s="1">
+      <c r="GP7" s="1">
         <f t="shared" si="3"/>
         <v>196</v>
       </c>
-      <c r="GQ3" s="1">
+      <c r="GQ7" s="1">
         <f t="shared" si="3"/>
         <v>197</v>
       </c>
-      <c r="GR3" s="1">
+      <c r="GR7" s="1">
         <f t="shared" si="3"/>
         <v>198</v>
       </c>
-      <c r="GS3" s="1">
+      <c r="GS7" s="1">
         <f t="shared" si="3"/>
         <v>199</v>
       </c>
-      <c r="GT3" s="1">
+      <c r="GT7" s="1">
         <f t="shared" si="3"/>
         <v>200</v>
       </c>
-      <c r="GU3" s="1">
+      <c r="GU7" s="1">
         <f t="shared" si="3"/>
         <v>201</v>
       </c>
-      <c r="GV3" s="1">
+      <c r="GV7" s="1">
         <f t="shared" si="3"/>
         <v>202</v>
       </c>
-      <c r="GW3" s="1">
+      <c r="GW7" s="1">
         <f t="shared" si="3"/>
         <v>203</v>
       </c>
-      <c r="GX3" s="1">
+      <c r="GX7" s="1">
         <f t="shared" si="3"/>
         <v>204</v>
       </c>
-      <c r="GY3" s="1">
+      <c r="GY7" s="1">
         <f t="shared" si="3"/>
         <v>205</v>
       </c>
-      <c r="GZ3" s="1">
+      <c r="GZ7" s="1">
         <f t="shared" si="3"/>
         <v>206</v>
       </c>
-      <c r="HA3" s="1">
+      <c r="HA7" s="1">
         <f t="shared" si="3"/>
         <v>207</v>
       </c>
-      <c r="HB3" s="1">
+      <c r="HB7" s="1">
         <f t="shared" si="3"/>
         <v>208</v>
       </c>
-      <c r="HC3" s="1">
+      <c r="HC7" s="1">
         <f t="shared" si="3"/>
         <v>209</v>
       </c>
-      <c r="HD3" s="1">
+      <c r="HD7" s="1">
         <f t="shared" si="3"/>
         <v>210</v>
       </c>
-      <c r="HE3" s="1">
+      <c r="HE7" s="1">
         <f t="shared" si="3"/>
         <v>211</v>
       </c>
-      <c r="HF3" s="1">
+      <c r="HF7" s="1">
         <f t="shared" si="3"/>
         <v>212</v>
       </c>
-      <c r="HG3" s="1">
+      <c r="HG7" s="1">
         <f t="shared" si="3"/>
         <v>213</v>
       </c>
-      <c r="HH3" s="1">
+      <c r="HH7" s="1">
         <f t="shared" si="3"/>
         <v>214</v>
       </c>
-      <c r="HI3" s="1">
+      <c r="HI7" s="1">
         <f t="shared" si="3"/>
         <v>215</v>
       </c>
-      <c r="HJ3" s="1">
+      <c r="HJ7" s="1">
         <f t="shared" si="3"/>
         <v>216</v>
       </c>
-      <c r="HK3" s="1">
+      <c r="HK7" s="1">
         <f t="shared" si="3"/>
         <v>217</v>
       </c>
-      <c r="HL3" s="1">
+      <c r="HL7" s="1">
         <f t="shared" si="3"/>
         <v>218</v>
       </c>
-      <c r="HM3" s="1">
+      <c r="HM7" s="1">
         <f t="shared" si="3"/>
         <v>219</v>
       </c>
-      <c r="HN3" s="1">
+      <c r="HN7" s="1">
         <f t="shared" si="3"/>
         <v>220</v>
       </c>
-      <c r="HO3" s="1">
+      <c r="HO7" s="1">
         <f t="shared" si="3"/>
         <v>221</v>
       </c>
-      <c r="HP3" s="1">
+      <c r="HP7" s="1">
         <f t="shared" si="3"/>
         <v>222</v>
       </c>
-      <c r="HQ3" s="1">
+      <c r="HQ7" s="1">
         <f t="shared" si="3"/>
         <v>223</v>
       </c>
-      <c r="HR3" s="1">
+      <c r="HR7" s="1">
         <f t="shared" si="3"/>
         <v>224</v>
       </c>
-      <c r="HS3" s="1">
+      <c r="HS7" s="1">
         <f t="shared" si="3"/>
         <v>225</v>
       </c>
-      <c r="HT3" s="1">
+      <c r="HT7" s="1">
         <f t="shared" si="3"/>
         <v>226</v>
       </c>
-      <c r="HU3" s="1">
+      <c r="HU7" s="1">
         <f t="shared" si="3"/>
         <v>227</v>
       </c>
-      <c r="HV3" s="1">
+      <c r="HV7" s="1">
         <f t="shared" si="3"/>
         <v>228</v>
       </c>
-      <c r="HW3" s="1">
+      <c r="HW7" s="1">
         <f t="shared" si="3"/>
         <v>229</v>
       </c>
-      <c r="HX3" s="1">
+      <c r="HX7" s="1">
         <f t="shared" si="3"/>
         <v>230</v>
       </c>
-      <c r="HY3" s="1">
+      <c r="HY7" s="1">
         <f t="shared" si="3"/>
         <v>231</v>
       </c>
-      <c r="HZ3" s="1">
+      <c r="HZ7" s="1">
         <f t="shared" si="3"/>
         <v>232</v>
       </c>
-      <c r="IA3" s="1">
+      <c r="IA7" s="1">
         <f t="shared" si="3"/>
         <v>233</v>
       </c>
-      <c r="IB3" s="1">
+      <c r="IB7" s="1">
         <f t="shared" si="3"/>
         <v>234</v>
       </c>
-      <c r="IC3" s="1">
+      <c r="IC7" s="1">
         <f t="shared" si="3"/>
         <v>235</v>
       </c>
-      <c r="ID3" s="1">
+      <c r="ID7" s="1">
         <f t="shared" si="3"/>
         <v>236</v>
       </c>
-      <c r="IE3" s="1">
+      <c r="IE7" s="1">
         <f t="shared" si="3"/>
         <v>237</v>
       </c>
-      <c r="IF3" s="1">
+      <c r="IF7" s="1">
         <f t="shared" si="3"/>
         <v>238</v>
       </c>
-      <c r="IG3" s="1">
+      <c r="IG7" s="1">
         <f t="shared" si="3"/>
         <v>239</v>
       </c>
-      <c r="IH3" s="1">
+      <c r="IH7" s="1">
         <f t="shared" si="3"/>
         <v>240</v>
       </c>
-      <c r="II3" s="1">
+      <c r="II7" s="1">
         <f t="shared" si="3"/>
         <v>241</v>
       </c>
-      <c r="IJ3" s="1">
+      <c r="IJ7" s="1">
         <f t="shared" si="3"/>
         <v>242</v>
       </c>
+      <c r="IK7" s="1">
+        <f t="shared" ref="IK7" si="4">IJ7+1</f>
+        <v>243</v>
+      </c>
+      <c r="IL7" s="1">
+        <f t="shared" ref="IL7" si="5">IK7+1</f>
+        <v>244</v>
+      </c>
+      <c r="IM7" s="1">
+        <f t="shared" ref="IM7" si="6">IL7+1</f>
+        <v>245</v>
+      </c>
+      <c r="IN7" s="1">
+        <f t="shared" ref="IN7" si="7">IM7+1</f>
+        <v>246</v>
+      </c>
+      <c r="IO7" s="1">
+        <f t="shared" ref="IO7" si="8">IN7+1</f>
+        <v>247</v>
+      </c>
+      <c r="IP7" s="1">
+        <f t="shared" ref="IP7" si="9">IO7+1</f>
+        <v>248</v>
+      </c>
+      <c r="IQ7" s="1">
+        <f t="shared" ref="IQ7" si="10">IP7+1</f>
+        <v>249</v>
+      </c>
+      <c r="IR7" s="1">
+        <f t="shared" ref="IR7" si="11">IQ7+1</f>
+        <v>250</v>
+      </c>
+      <c r="IS7" s="1">
+        <f t="shared" ref="IS7" si="12">IR7+1</f>
+        <v>251</v>
+      </c>
+      <c r="IT7" s="1">
+        <f t="shared" ref="IT7" si="13">IS7+1</f>
+        <v>252</v>
+      </c>
+      <c r="IU7" s="1">
+        <f t="shared" ref="IU7" si="14">IT7+1</f>
+        <v>253</v>
+      </c>
+      <c r="IV7" s="1">
+        <f t="shared" ref="IV7" si="15">IU7+1</f>
+        <v>254</v>
+      </c>
+      <c r="IW7" s="1">
+        <f t="shared" ref="IW7:IX7" si="16">IV7+1</f>
+        <v>255</v>
+      </c>
+      <c r="IX7" s="1">
+        <f t="shared" si="16"/>
+        <v>256</v>
+      </c>
     </row>
-    <row r="4" spans="1:244" x14ac:dyDescent="0.25">
-      <c r="B4" s="19"/>
-      <c r="C4" s="20"/>
-      <c r="D4" s="20"/>
-      <c r="E4" s="20"/>
-      <c r="F4" s="32"/>
-      <c r="G4" s="21" t="s">
-        <v>43</v>
-      </c>
-      <c r="H4" s="78" t="s">
-        <v>44</v>
-      </c>
-      <c r="I4" s="78"/>
-      <c r="J4" s="78"/>
-      <c r="K4" s="78"/>
-      <c r="L4" s="78"/>
-      <c r="M4" s="78"/>
-      <c r="N4" s="78"/>
-      <c r="O4" s="78"/>
-      <c r="P4" s="78"/>
-      <c r="Q4" s="78"/>
-      <c r="R4" s="78"/>
-      <c r="S4" s="79"/>
-      <c r="AJ4" s="80" t="s">
-        <v>55</v>
-      </c>
-      <c r="AK4" s="81" t="s">
-        <v>65</v>
-      </c>
-      <c r="AL4" s="81" t="s">
-        <v>56</v>
-      </c>
-      <c r="AM4" s="81"/>
-      <c r="AN4" s="81"/>
-      <c r="AO4" s="81"/>
-      <c r="AP4" s="81"/>
-      <c r="AQ4" s="81"/>
-      <c r="AR4" s="81" t="s">
-        <v>57</v>
-      </c>
-      <c r="AS4" s="81" t="s">
-        <v>56</v>
-      </c>
-      <c r="AT4" s="81"/>
-      <c r="AU4" s="81"/>
-      <c r="AV4" s="81"/>
-      <c r="AW4" s="48"/>
-      <c r="AX4" s="48"/>
-      <c r="AY4" s="81" t="s">
-        <v>68</v>
-      </c>
-      <c r="AZ4" s="81" t="s">
-        <v>58</v>
-      </c>
-      <c r="BA4" s="48"/>
-      <c r="BB4" s="84" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="5" spans="1:244" x14ac:dyDescent="0.25">
-      <c r="B5" s="22"/>
-      <c r="C5" s="23"/>
-      <c r="D5" s="23"/>
-      <c r="E5" s="23"/>
-      <c r="F5" s="33"/>
-      <c r="G5" s="21" t="s">
-        <v>43</v>
-      </c>
-      <c r="H5" s="78" t="s">
-        <v>45</v>
-      </c>
-      <c r="I5" s="78"/>
-      <c r="J5" s="78"/>
-      <c r="K5" s="78"/>
-      <c r="L5" s="78"/>
-      <c r="M5" s="78"/>
-      <c r="N5" s="78"/>
-      <c r="O5" s="78"/>
-      <c r="P5" s="78"/>
-      <c r="Q5" s="78"/>
-      <c r="R5" s="78"/>
-      <c r="S5" s="79"/>
-      <c r="AJ5" s="80"/>
-      <c r="AK5" s="81"/>
-      <c r="AL5" s="81"/>
-      <c r="AM5" s="81"/>
-      <c r="AN5" s="81"/>
-      <c r="AO5" s="81"/>
-      <c r="AP5" s="81"/>
-      <c r="AQ5" s="81"/>
-      <c r="AR5" s="81"/>
-      <c r="AS5" s="81"/>
-      <c r="AT5" s="81"/>
-      <c r="AU5" s="81"/>
-      <c r="AV5" s="81"/>
-      <c r="AW5" s="48"/>
-      <c r="AX5" s="48"/>
-      <c r="AY5" s="81"/>
-      <c r="AZ5" s="81"/>
-      <c r="BA5" s="48"/>
-      <c r="BB5" s="84"/>
-    </row>
-    <row r="6" spans="1:244" x14ac:dyDescent="0.25">
-      <c r="B6" s="43"/>
-      <c r="C6" s="44"/>
-      <c r="D6" s="44"/>
-      <c r="E6" s="44"/>
-      <c r="F6" s="45"/>
-      <c r="G6" s="21" t="s">
-        <v>43</v>
-      </c>
-      <c r="H6" s="78" t="s">
-        <v>54</v>
-      </c>
-      <c r="I6" s="78"/>
-      <c r="J6" s="78"/>
-      <c r="K6" s="78"/>
-      <c r="L6" s="78"/>
-      <c r="M6" s="78"/>
-      <c r="N6" s="78"/>
-      <c r="O6" s="78"/>
-      <c r="P6" s="78"/>
-      <c r="Q6" s="78"/>
-      <c r="R6" s="78"/>
-      <c r="S6" s="79"/>
-      <c r="AJ6" s="80"/>
-      <c r="AK6" s="81"/>
-      <c r="AL6" s="81"/>
-      <c r="AM6" s="81"/>
-      <c r="AN6" s="81"/>
-      <c r="AO6" s="81"/>
-      <c r="AP6" s="81"/>
-      <c r="AQ6" s="81"/>
-      <c r="AR6" s="81"/>
-      <c r="AS6" s="81"/>
-      <c r="AT6" s="81"/>
-      <c r="AU6" s="81"/>
-      <c r="AV6" s="81"/>
-      <c r="AW6" s="48"/>
-      <c r="AX6" s="48"/>
-      <c r="AY6" s="81"/>
-      <c r="AZ6" s="81"/>
-      <c r="BA6" s="48"/>
-      <c r="BB6" s="84"/>
-    </row>
-    <row r="7" spans="1:244" x14ac:dyDescent="0.25">
-      <c r="B7" s="38"/>
-      <c r="C7" s="39"/>
-      <c r="D7" s="39"/>
-      <c r="E7" s="39"/>
-      <c r="F7" s="40"/>
-      <c r="G7" s="21" t="s">
-        <v>43</v>
-      </c>
-      <c r="H7" s="78" t="s">
-        <v>53</v>
-      </c>
-      <c r="I7" s="78"/>
-      <c r="J7" s="78"/>
-      <c r="K7" s="78"/>
-      <c r="L7" s="78"/>
-      <c r="M7" s="78"/>
-      <c r="N7" s="78"/>
-      <c r="O7" s="78"/>
-      <c r="P7" s="78"/>
-      <c r="Q7" s="78"/>
-      <c r="R7" s="78"/>
-      <c r="S7" s="79"/>
-      <c r="AJ7" s="80"/>
-      <c r="AK7" s="81"/>
-      <c r="AL7" s="81"/>
-      <c r="AM7" s="81"/>
-      <c r="AN7" s="81"/>
-      <c r="AO7" s="81"/>
-      <c r="AP7" s="81"/>
-      <c r="AQ7" s="81"/>
-      <c r="AR7" s="81"/>
-      <c r="AS7" s="81"/>
-      <c r="AT7" s="81"/>
-      <c r="AU7" s="81"/>
-      <c r="AV7" s="81"/>
-      <c r="AW7" s="48"/>
-      <c r="AX7" s="48"/>
-      <c r="AY7" s="81"/>
-      <c r="AZ7" s="81"/>
-      <c r="BA7" s="48"/>
-      <c r="BB7" s="84"/>
-    </row>
-    <row r="8" spans="1:244" x14ac:dyDescent="0.25">
-      <c r="B8" s="24"/>
-      <c r="C8" s="25"/>
-      <c r="D8" s="25"/>
-      <c r="E8" s="25"/>
-      <c r="F8" s="34"/>
+    <row r="8" spans="1:258" x14ac:dyDescent="0.25">
+      <c r="B8" s="19"/>
+      <c r="C8" s="20"/>
+      <c r="D8" s="20"/>
+      <c r="E8" s="20"/>
+      <c r="F8" s="32"/>
       <c r="G8" s="21" t="s">
         <v>43</v>
       </c>
-      <c r="H8" s="78" t="s">
-        <v>46</v>
-      </c>
-      <c r="I8" s="78"/>
-      <c r="J8" s="78"/>
-      <c r="K8" s="78"/>
-      <c r="L8" s="78"/>
-      <c r="M8" s="78"/>
-      <c r="N8" s="78"/>
-      <c r="O8" s="78"/>
-      <c r="P8" s="78"/>
-      <c r="Q8" s="78"/>
-      <c r="R8" s="78"/>
-      <c r="S8" s="79"/>
-      <c r="AJ8" s="80"/>
-      <c r="AK8" s="81"/>
-      <c r="AL8" s="81"/>
-      <c r="AM8" s="81"/>
-      <c r="AN8" s="81"/>
-      <c r="AO8" s="81"/>
-      <c r="AP8" s="81"/>
-      <c r="AQ8" s="81"/>
-      <c r="AR8" s="81"/>
-      <c r="AS8" s="81"/>
-      <c r="AT8" s="81"/>
-      <c r="AU8" s="81"/>
-      <c r="AV8" s="81"/>
+      <c r="H8" s="82" t="s">
+        <v>44</v>
+      </c>
+      <c r="I8" s="82"/>
+      <c r="J8" s="82"/>
+      <c r="K8" s="82"/>
+      <c r="L8" s="82"/>
+      <c r="M8" s="82"/>
+      <c r="N8" s="82"/>
+      <c r="O8" s="82"/>
+      <c r="P8" s="82"/>
+      <c r="Q8" s="82"/>
+      <c r="R8" s="82"/>
+      <c r="S8" s="83"/>
+      <c r="AJ8" s="84" t="s">
+        <v>55</v>
+      </c>
+      <c r="AK8" s="85" t="s">
+        <v>65</v>
+      </c>
+      <c r="AL8" s="85" t="s">
+        <v>56</v>
+      </c>
+      <c r="AM8" s="85"/>
+      <c r="AN8" s="85"/>
+      <c r="AO8" s="85"/>
+      <c r="AP8" s="85"/>
+      <c r="AQ8" s="85"/>
+      <c r="AR8" s="85" t="s">
+        <v>57</v>
+      </c>
+      <c r="AS8" s="85" t="s">
+        <v>56</v>
+      </c>
+      <c r="AT8" s="85"/>
+      <c r="AU8" s="85"/>
+      <c r="AV8" s="85"/>
       <c r="AW8" s="48"/>
       <c r="AX8" s="48"/>
-      <c r="AY8" s="81"/>
-      <c r="AZ8" s="81"/>
+      <c r="AY8" s="85" t="s">
+        <v>68</v>
+      </c>
+      <c r="AZ8" s="85" t="s">
+        <v>58</v>
+      </c>
       <c r="BA8" s="48"/>
-      <c r="BB8" s="84"/>
+      <c r="BB8" s="88" t="s">
+        <v>59</v>
+      </c>
     </row>
-    <row r="9" spans="1:244" x14ac:dyDescent="0.25">
-      <c r="B9" s="26"/>
-      <c r="C9" s="27"/>
-      <c r="D9" s="27"/>
-      <c r="E9" s="27"/>
-      <c r="F9" s="35"/>
+    <row r="9" spans="1:258" x14ac:dyDescent="0.25">
+      <c r="B9" s="22"/>
+      <c r="C9" s="23"/>
+      <c r="D9" s="23"/>
+      <c r="E9" s="23"/>
+      <c r="F9" s="33"/>
       <c r="G9" s="21" t="s">
         <v>43</v>
       </c>
-      <c r="H9" s="78" t="s">
-        <v>47</v>
-      </c>
-      <c r="I9" s="78"/>
-      <c r="J9" s="78"/>
-      <c r="K9" s="78"/>
-      <c r="L9" s="78"/>
-      <c r="M9" s="78"/>
-      <c r="N9" s="78"/>
-      <c r="O9" s="78"/>
-      <c r="P9" s="78"/>
-      <c r="Q9" s="78"/>
-      <c r="R9" s="78"/>
-      <c r="S9" s="79"/>
-      <c r="AJ9" s="80"/>
-      <c r="AK9" s="81"/>
-      <c r="AL9" s="81"/>
-      <c r="AM9" s="81"/>
-      <c r="AN9" s="81"/>
-      <c r="AO9" s="81"/>
-      <c r="AP9" s="81"/>
-      <c r="AQ9" s="81"/>
-      <c r="AR9" s="81"/>
-      <c r="AS9" s="81"/>
-      <c r="AT9" s="81"/>
-      <c r="AU9" s="81"/>
-      <c r="AV9" s="81"/>
+      <c r="H9" s="82" t="s">
+        <v>45</v>
+      </c>
+      <c r="I9" s="82"/>
+      <c r="J9" s="82"/>
+      <c r="K9" s="82"/>
+      <c r="L9" s="82"/>
+      <c r="M9" s="82"/>
+      <c r="N9" s="82"/>
+      <c r="O9" s="82"/>
+      <c r="P9" s="82"/>
+      <c r="Q9" s="82"/>
+      <c r="R9" s="82"/>
+      <c r="S9" s="83"/>
+      <c r="AJ9" s="84"/>
+      <c r="AK9" s="85"/>
+      <c r="AL9" s="85"/>
+      <c r="AM9" s="85"/>
+      <c r="AN9" s="85"/>
+      <c r="AO9" s="85"/>
+      <c r="AP9" s="85"/>
+      <c r="AQ9" s="85"/>
+      <c r="AR9" s="85"/>
+      <c r="AS9" s="85"/>
+      <c r="AT9" s="85"/>
+      <c r="AU9" s="85"/>
+      <c r="AV9" s="85"/>
       <c r="AW9" s="48"/>
       <c r="AX9" s="48"/>
-      <c r="AY9" s="81"/>
-      <c r="AZ9" s="81"/>
+      <c r="AY9" s="85"/>
+      <c r="AZ9" s="85"/>
       <c r="BA9" s="48"/>
-      <c r="BB9" s="84"/>
+      <c r="BB9" s="88"/>
     </row>
-    <row r="10" spans="1:244" x14ac:dyDescent="0.25">
-      <c r="B10" s="28"/>
-      <c r="C10" s="29"/>
-      <c r="D10" s="29"/>
-      <c r="E10" s="29"/>
-      <c r="F10" s="36"/>
+    <row r="10" spans="1:258" x14ac:dyDescent="0.25">
+      <c r="B10" s="43"/>
+      <c r="C10" s="44"/>
+      <c r="D10" s="44"/>
+      <c r="E10" s="44"/>
+      <c r="F10" s="45"/>
       <c r="G10" s="21" t="s">
         <v>43</v>
       </c>
-      <c r="H10" s="78" t="s">
-        <v>48</v>
-      </c>
-      <c r="I10" s="78"/>
-      <c r="J10" s="78"/>
-      <c r="K10" s="78"/>
-      <c r="L10" s="78"/>
-      <c r="M10" s="78"/>
-      <c r="N10" s="78"/>
-      <c r="O10" s="78"/>
-      <c r="P10" s="78"/>
-      <c r="Q10" s="78"/>
-      <c r="R10" s="78"/>
-      <c r="S10" s="79"/>
-      <c r="AJ10" s="80"/>
-      <c r="AK10" s="81"/>
-      <c r="AL10" s="81"/>
-      <c r="AM10" s="81"/>
-      <c r="AN10" s="81"/>
-      <c r="AO10" s="81"/>
-      <c r="AP10" s="81"/>
-      <c r="AQ10" s="81"/>
-      <c r="AR10" s="81"/>
-      <c r="AS10" s="81"/>
-      <c r="AT10" s="81"/>
-      <c r="AU10" s="81"/>
-      <c r="AV10" s="81"/>
+      <c r="H10" s="82" t="s">
+        <v>54</v>
+      </c>
+      <c r="I10" s="82"/>
+      <c r="J10" s="82"/>
+      <c r="K10" s="82"/>
+      <c r="L10" s="82"/>
+      <c r="M10" s="82"/>
+      <c r="N10" s="82"/>
+      <c r="O10" s="82"/>
+      <c r="P10" s="82"/>
+      <c r="Q10" s="82"/>
+      <c r="R10" s="82"/>
+      <c r="S10" s="83"/>
+      <c r="AJ10" s="84"/>
+      <c r="AK10" s="85"/>
+      <c r="AL10" s="85"/>
+      <c r="AM10" s="85"/>
+      <c r="AN10" s="85"/>
+      <c r="AO10" s="85"/>
+      <c r="AP10" s="85"/>
+      <c r="AQ10" s="85"/>
+      <c r="AR10" s="85"/>
+      <c r="AS10" s="85"/>
+      <c r="AT10" s="85"/>
+      <c r="AU10" s="85"/>
+      <c r="AV10" s="85"/>
       <c r="AW10" s="48"/>
       <c r="AX10" s="48"/>
-      <c r="AY10" s="81"/>
-      <c r="AZ10" s="81"/>
+      <c r="AY10" s="85"/>
+      <c r="AZ10" s="85"/>
       <c r="BA10" s="48"/>
-      <c r="BB10" s="84"/>
+      <c r="BB10" s="88"/>
     </row>
-    <row r="11" spans="1:244" x14ac:dyDescent="0.25">
-      <c r="B11" s="30"/>
-      <c r="C11" s="31"/>
-      <c r="D11" s="31"/>
-      <c r="E11" s="31"/>
-      <c r="F11" s="37"/>
+    <row r="11" spans="1:258" x14ac:dyDescent="0.25">
+      <c r="B11" s="38"/>
+      <c r="C11" s="39"/>
+      <c r="D11" s="39"/>
+      <c r="E11" s="39"/>
+      <c r="F11" s="40"/>
       <c r="G11" s="21" t="s">
         <v>43</v>
       </c>
-      <c r="H11" s="78" t="s">
-        <v>49</v>
-      </c>
-      <c r="I11" s="78"/>
-      <c r="J11" s="78"/>
-      <c r="K11" s="78"/>
-      <c r="L11" s="78"/>
-      <c r="M11" s="78"/>
-      <c r="N11" s="78"/>
-      <c r="O11" s="78"/>
-      <c r="P11" s="78"/>
-      <c r="Q11" s="78"/>
-      <c r="R11" s="78"/>
-      <c r="S11" s="79"/>
-      <c r="AJ11" s="80"/>
-      <c r="AK11" s="81"/>
-      <c r="AL11" s="81"/>
-      <c r="AM11" s="81"/>
-      <c r="AN11" s="81"/>
-      <c r="AO11" s="81"/>
-      <c r="AP11" s="81"/>
-      <c r="AQ11" s="81"/>
-      <c r="AR11" s="81"/>
-      <c r="AS11" s="81"/>
-      <c r="AT11" s="81"/>
-      <c r="AU11" s="81"/>
-      <c r="AV11" s="81"/>
+      <c r="H11" s="82" t="s">
+        <v>53</v>
+      </c>
+      <c r="I11" s="82"/>
+      <c r="J11" s="82"/>
+      <c r="K11" s="82"/>
+      <c r="L11" s="82"/>
+      <c r="M11" s="82"/>
+      <c r="N11" s="82"/>
+      <c r="O11" s="82"/>
+      <c r="P11" s="82"/>
+      <c r="Q11" s="82"/>
+      <c r="R11" s="82"/>
+      <c r="S11" s="83"/>
+      <c r="AJ11" s="84"/>
+      <c r="AK11" s="85"/>
+      <c r="AL11" s="85"/>
+      <c r="AM11" s="85"/>
+      <c r="AN11" s="85"/>
+      <c r="AO11" s="85"/>
+      <c r="AP11" s="85"/>
+      <c r="AQ11" s="85"/>
+      <c r="AR11" s="85"/>
+      <c r="AS11" s="85"/>
+      <c r="AT11" s="85"/>
+      <c r="AU11" s="85"/>
+      <c r="AV11" s="85"/>
       <c r="AW11" s="48"/>
       <c r="AX11" s="48"/>
-      <c r="AY11" s="81"/>
-      <c r="AZ11" s="81"/>
+      <c r="AY11" s="85"/>
+      <c r="AZ11" s="85"/>
       <c r="BA11" s="48"/>
-      <c r="BB11" s="84"/>
+      <c r="BB11" s="88"/>
     </row>
-    <row r="12" spans="1:244" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B12" s="57"/>
-      <c r="C12" s="58"/>
-      <c r="D12" s="58"/>
-      <c r="E12" s="58"/>
-      <c r="F12" s="59"/>
+    <row r="12" spans="1:258" x14ac:dyDescent="0.25">
+      <c r="B12" s="24"/>
+      <c r="C12" s="25"/>
+      <c r="D12" s="25"/>
+      <c r="E12" s="25"/>
+      <c r="F12" s="34"/>
       <c r="G12" s="21" t="s">
         <v>43</v>
       </c>
-      <c r="H12" s="78" t="s">
-        <v>50</v>
-      </c>
-      <c r="I12" s="78"/>
-      <c r="J12" s="78"/>
-      <c r="K12" s="78"/>
-      <c r="L12" s="78"/>
-      <c r="M12" s="78"/>
-      <c r="N12" s="78"/>
-      <c r="O12" s="78"/>
-      <c r="P12" s="78"/>
-      <c r="Q12" s="78"/>
-      <c r="R12" s="78"/>
-      <c r="S12" s="79"/>
-      <c r="AJ12" s="80"/>
-      <c r="AK12" s="81"/>
-      <c r="AL12" s="81"/>
-      <c r="AM12" s="81"/>
-      <c r="AN12" s="81"/>
-      <c r="AO12" s="81"/>
-      <c r="AP12" s="81"/>
-      <c r="AQ12" s="81"/>
-      <c r="AR12" s="81"/>
-      <c r="AS12" s="81"/>
-      <c r="AT12" s="81"/>
-      <c r="AU12" s="81"/>
-      <c r="AV12" s="81"/>
+      <c r="H12" s="82" t="s">
+        <v>46</v>
+      </c>
+      <c r="I12" s="82"/>
+      <c r="J12" s="82"/>
+      <c r="K12" s="82"/>
+      <c r="L12" s="82"/>
+      <c r="M12" s="82"/>
+      <c r="N12" s="82"/>
+      <c r="O12" s="82"/>
+      <c r="P12" s="82"/>
+      <c r="Q12" s="82"/>
+      <c r="R12" s="82"/>
+      <c r="S12" s="83"/>
+      <c r="AJ12" s="84"/>
+      <c r="AK12" s="85"/>
+      <c r="AL12" s="85"/>
+      <c r="AM12" s="85"/>
+      <c r="AN12" s="85"/>
+      <c r="AO12" s="85"/>
+      <c r="AP12" s="85"/>
+      <c r="AQ12" s="85"/>
+      <c r="AR12" s="85"/>
+      <c r="AS12" s="85"/>
+      <c r="AT12" s="85"/>
+      <c r="AU12" s="85"/>
+      <c r="AV12" s="85"/>
       <c r="AW12" s="48"/>
       <c r="AX12" s="48"/>
-      <c r="AY12" s="81"/>
-      <c r="AZ12" s="81"/>
+      <c r="AY12" s="85"/>
+      <c r="AZ12" s="85"/>
       <c r="BA12" s="48"/>
-      <c r="BB12" s="84"/>
+      <c r="BB12" s="88"/>
     </row>
-    <row r="13" spans="1:244" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B13" s="60"/>
-      <c r="C13" s="61"/>
-      <c r="D13" s="61"/>
-      <c r="E13" s="61"/>
-      <c r="F13" s="62"/>
+    <row r="13" spans="1:258" x14ac:dyDescent="0.25">
+      <c r="B13" s="26"/>
+      <c r="C13" s="27"/>
+      <c r="D13" s="27"/>
+      <c r="E13" s="27"/>
+      <c r="F13" s="35"/>
       <c r="G13" s="21" t="s">
         <v>43</v>
       </c>
-      <c r="H13" s="78" t="s">
-        <v>66</v>
-      </c>
-      <c r="I13" s="78"/>
-      <c r="J13" s="78"/>
-      <c r="K13" s="78"/>
-      <c r="L13" s="78"/>
-      <c r="M13" s="78"/>
-      <c r="N13" s="78"/>
-      <c r="O13" s="78"/>
-      <c r="P13" s="78"/>
-      <c r="Q13" s="78"/>
-      <c r="R13" s="78"/>
-      <c r="S13" s="79"/>
-      <c r="AJ13" s="72" t="s">
-        <v>60</v>
-      </c>
-      <c r="AK13" s="73"/>
-      <c r="AL13" s="73"/>
-      <c r="AM13" s="73"/>
-      <c r="AN13" s="73"/>
-      <c r="AO13" s="73"/>
-      <c r="AP13" s="73"/>
-      <c r="AQ13" s="73"/>
-      <c r="AR13" s="73"/>
-      <c r="AS13" s="73"/>
-      <c r="AT13" s="73"/>
-      <c r="AU13" s="73"/>
-      <c r="AV13" s="73"/>
-      <c r="AW13" s="73"/>
-      <c r="AX13" s="73"/>
-      <c r="AY13" s="73"/>
-      <c r="AZ13" s="73"/>
-      <c r="BA13" s="73"/>
-      <c r="BB13" s="74"/>
+      <c r="H13" s="82" t="s">
+        <v>47</v>
+      </c>
+      <c r="I13" s="82"/>
+      <c r="J13" s="82"/>
+      <c r="K13" s="82"/>
+      <c r="L13" s="82"/>
+      <c r="M13" s="82"/>
+      <c r="N13" s="82"/>
+      <c r="O13" s="82"/>
+      <c r="P13" s="82"/>
+      <c r="Q13" s="82"/>
+      <c r="R13" s="82"/>
+      <c r="S13" s="83"/>
+      <c r="AJ13" s="84"/>
+      <c r="AK13" s="85"/>
+      <c r="AL13" s="85"/>
+      <c r="AM13" s="85"/>
+      <c r="AN13" s="85"/>
+      <c r="AO13" s="85"/>
+      <c r="AP13" s="85"/>
+      <c r="AQ13" s="85"/>
+      <c r="AR13" s="85"/>
+      <c r="AS13" s="85"/>
+      <c r="AT13" s="85"/>
+      <c r="AU13" s="85"/>
+      <c r="AV13" s="85"/>
+      <c r="AW13" s="48"/>
+      <c r="AX13" s="48"/>
+      <c r="AY13" s="85"/>
+      <c r="AZ13" s="85"/>
+      <c r="BA13" s="48"/>
+      <c r="BB13" s="88"/>
     </row>
-    <row r="14" spans="1:244" x14ac:dyDescent="0.25">
-      <c r="B14" s="63"/>
-      <c r="C14" s="64"/>
-      <c r="D14" s="64"/>
-      <c r="E14" s="64"/>
-      <c r="F14" s="65"/>
+    <row r="14" spans="1:258" x14ac:dyDescent="0.25">
+      <c r="B14" s="28"/>
+      <c r="C14" s="29"/>
+      <c r="D14" s="29"/>
+      <c r="E14" s="29"/>
+      <c r="F14" s="36"/>
       <c r="G14" s="21" t="s">
         <v>43</v>
       </c>
-      <c r="H14" s="78" t="s">
-        <v>67</v>
-      </c>
-      <c r="I14" s="78"/>
-      <c r="J14" s="78"/>
-      <c r="K14" s="78"/>
-      <c r="L14" s="78"/>
-      <c r="M14" s="78"/>
-      <c r="N14" s="78"/>
-      <c r="O14" s="78"/>
-      <c r="P14" s="78"/>
-      <c r="Q14" s="78"/>
-      <c r="R14" s="78"/>
-      <c r="S14" s="79"/>
-      <c r="AJ14" s="55"/>
-      <c r="AK14" s="55"/>
-      <c r="AL14" s="55"/>
-      <c r="AM14" s="55"/>
-      <c r="AN14" s="55"/>
-      <c r="AO14" s="55"/>
-      <c r="AP14" s="55"/>
-      <c r="AQ14" s="55"/>
-      <c r="AR14" s="55"/>
-      <c r="AS14" s="55"/>
-      <c r="AT14" s="55"/>
-      <c r="AU14" s="55"/>
-      <c r="AV14" s="55"/>
+      <c r="H14" s="82" t="s">
+        <v>48</v>
+      </c>
+      <c r="I14" s="82"/>
+      <c r="J14" s="82"/>
+      <c r="K14" s="82"/>
+      <c r="L14" s="82"/>
+      <c r="M14" s="82"/>
+      <c r="N14" s="82"/>
+      <c r="O14" s="82"/>
+      <c r="P14" s="82"/>
+      <c r="Q14" s="82"/>
+      <c r="R14" s="82"/>
+      <c r="S14" s="83"/>
+      <c r="AJ14" s="84"/>
+      <c r="AK14" s="85"/>
+      <c r="AL14" s="85"/>
+      <c r="AM14" s="85"/>
+      <c r="AN14" s="85"/>
+      <c r="AO14" s="85"/>
+      <c r="AP14" s="85"/>
+      <c r="AQ14" s="85"/>
+      <c r="AR14" s="85"/>
+      <c r="AS14" s="85"/>
+      <c r="AT14" s="85"/>
+      <c r="AU14" s="85"/>
+      <c r="AV14" s="85"/>
       <c r="AW14" s="48"/>
       <c r="AX14" s="48"/>
-      <c r="AY14" s="48"/>
-      <c r="AZ14" s="55"/>
+      <c r="AY14" s="85"/>
+      <c r="AZ14" s="85"/>
       <c r="BA14" s="48"/>
-      <c r="BB14" s="55"/>
+      <c r="BB14" s="88"/>
     </row>
-    <row r="15" spans="1:244" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="16" spans="1:244" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B16" s="75" t="s">
+    <row r="15" spans="1:258" x14ac:dyDescent="0.25">
+      <c r="B15" s="30"/>
+      <c r="C15" s="31"/>
+      <c r="D15" s="31"/>
+      <c r="E15" s="31"/>
+      <c r="F15" s="37"/>
+      <c r="G15" s="21" t="s">
+        <v>43</v>
+      </c>
+      <c r="H15" s="82" t="s">
+        <v>49</v>
+      </c>
+      <c r="I15" s="82"/>
+      <c r="J15" s="82"/>
+      <c r="K15" s="82"/>
+      <c r="L15" s="82"/>
+      <c r="M15" s="82"/>
+      <c r="N15" s="82"/>
+      <c r="O15" s="82"/>
+      <c r="P15" s="82"/>
+      <c r="Q15" s="82"/>
+      <c r="R15" s="82"/>
+      <c r="S15" s="83"/>
+      <c r="AJ15" s="84"/>
+      <c r="AK15" s="85"/>
+      <c r="AL15" s="85"/>
+      <c r="AM15" s="85"/>
+      <c r="AN15" s="85"/>
+      <c r="AO15" s="85"/>
+      <c r="AP15" s="85"/>
+      <c r="AQ15" s="85"/>
+      <c r="AR15" s="85"/>
+      <c r="AS15" s="85"/>
+      <c r="AT15" s="85"/>
+      <c r="AU15" s="85"/>
+      <c r="AV15" s="85"/>
+      <c r="AW15" s="48"/>
+      <c r="AX15" s="48"/>
+      <c r="AY15" s="85"/>
+      <c r="AZ15" s="85"/>
+      <c r="BA15" s="48"/>
+      <c r="BB15" s="88"/>
+    </row>
+    <row r="16" spans="1:258" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B16" s="56"/>
+      <c r="C16" s="57"/>
+      <c r="D16" s="57"/>
+      <c r="E16" s="57"/>
+      <c r="F16" s="58"/>
+      <c r="G16" s="21" t="s">
+        <v>43</v>
+      </c>
+      <c r="H16" s="82" t="s">
+        <v>50</v>
+      </c>
+      <c r="I16" s="82"/>
+      <c r="J16" s="82"/>
+      <c r="K16" s="82"/>
+      <c r="L16" s="82"/>
+      <c r="M16" s="82"/>
+      <c r="N16" s="82"/>
+      <c r="O16" s="82"/>
+      <c r="P16" s="82"/>
+      <c r="Q16" s="82"/>
+      <c r="R16" s="82"/>
+      <c r="S16" s="83"/>
+      <c r="AJ16" s="84"/>
+      <c r="AK16" s="85"/>
+      <c r="AL16" s="85"/>
+      <c r="AM16" s="85"/>
+      <c r="AN16" s="85"/>
+      <c r="AO16" s="85"/>
+      <c r="AP16" s="85"/>
+      <c r="AQ16" s="85"/>
+      <c r="AR16" s="85"/>
+      <c r="AS16" s="85"/>
+      <c r="AT16" s="85"/>
+      <c r="AU16" s="85"/>
+      <c r="AV16" s="85"/>
+      <c r="AW16" s="48"/>
+      <c r="AX16" s="48"/>
+      <c r="AY16" s="85"/>
+      <c r="AZ16" s="85"/>
+      <c r="BA16" s="48"/>
+      <c r="BB16" s="88"/>
+    </row>
+    <row r="17" spans="2:54" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B17" s="59"/>
+      <c r="C17" s="60"/>
+      <c r="D17" s="60"/>
+      <c r="E17" s="60"/>
+      <c r="F17" s="61"/>
+      <c r="G17" s="21" t="s">
+        <v>43</v>
+      </c>
+      <c r="H17" s="82" t="s">
+        <v>66</v>
+      </c>
+      <c r="I17" s="82"/>
+      <c r="J17" s="82"/>
+      <c r="K17" s="82"/>
+      <c r="L17" s="82"/>
+      <c r="M17" s="82"/>
+      <c r="N17" s="82"/>
+      <c r="O17" s="82"/>
+      <c r="P17" s="82"/>
+      <c r="Q17" s="82"/>
+      <c r="R17" s="82"/>
+      <c r="S17" s="83"/>
+      <c r="AJ17" s="76" t="s">
+        <v>60</v>
+      </c>
+      <c r="AK17" s="77"/>
+      <c r="AL17" s="77"/>
+      <c r="AM17" s="77"/>
+      <c r="AN17" s="77"/>
+      <c r="AO17" s="77"/>
+      <c r="AP17" s="77"/>
+      <c r="AQ17" s="77"/>
+      <c r="AR17" s="77"/>
+      <c r="AS17" s="77"/>
+      <c r="AT17" s="77"/>
+      <c r="AU17" s="77"/>
+      <c r="AV17" s="77"/>
+      <c r="AW17" s="77"/>
+      <c r="AX17" s="77"/>
+      <c r="AY17" s="77"/>
+      <c r="AZ17" s="77"/>
+      <c r="BA17" s="77"/>
+      <c r="BB17" s="78"/>
+    </row>
+    <row r="18" spans="2:54" x14ac:dyDescent="0.25">
+      <c r="B18" s="62"/>
+      <c r="C18" s="63"/>
+      <c r="D18" s="63"/>
+      <c r="E18" s="63"/>
+      <c r="F18" s="64"/>
+      <c r="G18" s="21" t="s">
+        <v>43</v>
+      </c>
+      <c r="H18" s="82" t="s">
+        <v>67</v>
+      </c>
+      <c r="I18" s="82"/>
+      <c r="J18" s="82"/>
+      <c r="K18" s="82"/>
+      <c r="L18" s="82"/>
+      <c r="M18" s="82"/>
+      <c r="N18" s="82"/>
+      <c r="O18" s="82"/>
+      <c r="P18" s="82"/>
+      <c r="Q18" s="82"/>
+      <c r="R18" s="82"/>
+      <c r="S18" s="83"/>
+      <c r="AJ18" s="55"/>
+      <c r="AK18" s="55"/>
+      <c r="AL18" s="55"/>
+      <c r="AM18" s="55"/>
+      <c r="AN18" s="55"/>
+      <c r="AO18" s="55"/>
+      <c r="AP18" s="55"/>
+      <c r="AQ18" s="55"/>
+      <c r="AR18" s="55"/>
+      <c r="AS18" s="55"/>
+      <c r="AT18" s="55"/>
+      <c r="AU18" s="55"/>
+      <c r="AV18" s="55"/>
+      <c r="AW18" s="48"/>
+      <c r="AX18" s="48"/>
+      <c r="AY18" s="48"/>
+      <c r="AZ18" s="55"/>
+      <c r="BA18" s="48"/>
+      <c r="BB18" s="55"/>
+    </row>
+    <row r="19" spans="2:54" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="20" spans="2:54" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B20" s="79" t="s">
         <v>69</v>
       </c>
-      <c r="C16" s="76"/>
-      <c r="D16" s="76"/>
-      <c r="E16" s="76"/>
-      <c r="F16" s="76"/>
-      <c r="G16" s="76"/>
-      <c r="H16" s="76"/>
-      <c r="I16" s="76"/>
-      <c r="J16" s="76"/>
-      <c r="K16" s="76"/>
-      <c r="L16" s="76"/>
-      <c r="M16" s="76"/>
-      <c r="N16" s="76"/>
-      <c r="O16" s="76"/>
-      <c r="P16" s="76"/>
-      <c r="Q16" s="76"/>
-      <c r="R16" s="76"/>
-      <c r="S16" s="77"/>
+      <c r="C20" s="80"/>
+      <c r="D20" s="80"/>
+      <c r="E20" s="80"/>
+      <c r="F20" s="80"/>
+      <c r="G20" s="80"/>
+      <c r="H20" s="80"/>
+      <c r="I20" s="80"/>
+      <c r="J20" s="80"/>
+      <c r="K20" s="80"/>
+      <c r="L20" s="80"/>
+      <c r="M20" s="80"/>
+      <c r="N20" s="80"/>
+      <c r="O20" s="80"/>
+      <c r="P20" s="80"/>
+      <c r="Q20" s="80"/>
+      <c r="R20" s="80"/>
+      <c r="S20" s="81"/>
     </row>
-    <row r="17" spans="2:19" x14ac:dyDescent="0.25">
-      <c r="B17" s="47" t="s">
+    <row r="21" spans="2:54" x14ac:dyDescent="0.25">
+      <c r="B21" s="47" t="s">
         <v>62</v>
       </c>
-      <c r="C17" s="48"/>
-      <c r="D17" s="48"/>
-      <c r="E17" s="48"/>
-      <c r="F17" s="54" t="s">
-        <v>61</v>
-      </c>
-      <c r="G17" s="48"/>
-      <c r="H17" s="48"/>
-      <c r="I17" s="48"/>
-      <c r="J17" s="48"/>
-      <c r="K17" s="48"/>
-      <c r="L17" s="48"/>
-      <c r="M17" s="48"/>
-      <c r="N17" s="48"/>
-      <c r="O17" s="48"/>
-      <c r="P17" s="48"/>
-      <c r="Q17" s="48"/>
-      <c r="R17" s="48"/>
-      <c r="S17" s="49"/>
-    </row>
-    <row r="18" spans="2:19" x14ac:dyDescent="0.25">
-      <c r="B18" s="47" t="s">
-        <v>63</v>
-      </c>
-      <c r="C18" s="48"/>
-      <c r="D18" s="48"/>
-      <c r="E18" s="48"/>
-      <c r="F18" s="53">
-        <v>254</v>
-      </c>
-      <c r="G18" s="48"/>
-      <c r="H18" s="48"/>
-      <c r="I18" s="48"/>
-      <c r="J18" s="48"/>
-      <c r="K18" s="48"/>
-      <c r="L18" s="48"/>
-      <c r="M18" s="48"/>
-      <c r="N18" s="48"/>
-      <c r="O18" s="48"/>
-      <c r="P18" s="48"/>
-      <c r="Q18" s="48"/>
-      <c r="R18" s="48"/>
-      <c r="S18" s="49"/>
-    </row>
-    <row r="19" spans="2:19" x14ac:dyDescent="0.25">
-      <c r="B19" s="47"/>
-      <c r="C19" s="48"/>
-      <c r="D19" s="48"/>
-      <c r="E19" s="48"/>
-      <c r="F19" s="48"/>
-      <c r="G19" s="48"/>
-      <c r="H19" s="48"/>
-      <c r="I19" s="48"/>
-      <c r="J19" s="48"/>
-      <c r="K19" s="48"/>
-      <c r="L19" s="48"/>
-      <c r="M19" s="48"/>
-      <c r="N19" s="48"/>
-      <c r="O19" s="48"/>
-      <c r="P19" s="48"/>
-      <c r="Q19" s="48"/>
-      <c r="R19" s="48"/>
-      <c r="S19" s="49"/>
-    </row>
-    <row r="20" spans="2:19" x14ac:dyDescent="0.25">
-      <c r="B20" s="47" t="s">
-        <v>64</v>
-      </c>
-      <c r="C20" s="48"/>
-      <c r="D20" s="48"/>
-      <c r="E20" s="48"/>
-      <c r="F20" s="48"/>
-      <c r="G20" s="48"/>
-      <c r="H20" s="48"/>
-      <c r="I20" s="48"/>
-      <c r="J20" s="48"/>
-      <c r="K20" s="48"/>
-      <c r="L20" s="48"/>
-      <c r="M20" s="48"/>
-      <c r="N20" s="48"/>
-      <c r="O20" s="48"/>
-      <c r="P20" s="48"/>
-      <c r="Q20" s="48"/>
-      <c r="R20" s="48"/>
-      <c r="S20" s="49"/>
-    </row>
-    <row r="21" spans="2:19" x14ac:dyDescent="0.25">
-      <c r="B21" s="47"/>
       <c r="C21" s="48"/>
       <c r="D21" s="48"/>
       <c r="E21" s="48"/>
-      <c r="F21" s="48"/>
+      <c r="F21" s="54" t="s">
+        <v>61</v>
+      </c>
       <c r="G21" s="48"/>
       <c r="H21" s="48"/>
       <c r="I21" s="48"/>
@@ -3930,52 +5925,151 @@
       <c r="R21" s="48"/>
       <c r="S21" s="49"/>
     </row>
-    <row r="22" spans="2:19" x14ac:dyDescent="0.25">
-      <c r="B22" s="50" t="s">
+    <row r="22" spans="2:54" x14ac:dyDescent="0.25">
+      <c r="B22" s="47" t="s">
+        <v>63</v>
+      </c>
+      <c r="C22" s="48"/>
+      <c r="D22" s="48"/>
+      <c r="E22" s="48"/>
+      <c r="F22" s="53">
+        <v>254</v>
+      </c>
+      <c r="G22" s="48"/>
+      <c r="H22" s="48"/>
+      <c r="I22" s="48"/>
+      <c r="J22" s="48"/>
+      <c r="K22" s="48"/>
+      <c r="L22" s="48"/>
+      <c r="M22" s="48"/>
+      <c r="N22" s="48"/>
+      <c r="O22" s="48"/>
+      <c r="P22" s="48"/>
+      <c r="Q22" s="48"/>
+      <c r="R22" s="48"/>
+      <c r="S22" s="49"/>
+    </row>
+    <row r="23" spans="2:54" x14ac:dyDescent="0.25">
+      <c r="B23" s="47"/>
+      <c r="C23" s="48"/>
+      <c r="D23" s="48"/>
+      <c r="E23" s="48"/>
+      <c r="F23" s="48"/>
+      <c r="G23" s="48"/>
+      <c r="H23" s="48"/>
+      <c r="I23" s="48"/>
+      <c r="J23" s="48"/>
+      <c r="K23" s="48"/>
+      <c r="L23" s="48"/>
+      <c r="M23" s="48"/>
+      <c r="N23" s="48"/>
+      <c r="O23" s="48"/>
+      <c r="P23" s="48"/>
+      <c r="Q23" s="48"/>
+      <c r="R23" s="48"/>
+      <c r="S23" s="49"/>
+    </row>
+    <row r="24" spans="2:54" x14ac:dyDescent="0.25">
+      <c r="B24" s="47" t="s">
+        <v>64</v>
+      </c>
+      <c r="C24" s="48"/>
+      <c r="D24" s="48"/>
+      <c r="E24" s="48"/>
+      <c r="F24" s="48"/>
+      <c r="G24" s="48"/>
+      <c r="H24" s="48"/>
+      <c r="I24" s="48"/>
+      <c r="J24" s="48"/>
+      <c r="K24" s="48"/>
+      <c r="L24" s="48"/>
+      <c r="M24" s="48"/>
+      <c r="N24" s="48"/>
+      <c r="O24" s="48"/>
+      <c r="P24" s="48"/>
+      <c r="Q24" s="48"/>
+      <c r="R24" s="48"/>
+      <c r="S24" s="49"/>
+    </row>
+    <row r="25" spans="2:54" x14ac:dyDescent="0.25">
+      <c r="B25" s="47"/>
+      <c r="C25" s="48"/>
+      <c r="D25" s="48"/>
+      <c r="E25" s="48"/>
+      <c r="F25" s="48"/>
+      <c r="G25" s="48"/>
+      <c r="H25" s="48"/>
+      <c r="I25" s="48"/>
+      <c r="J25" s="48"/>
+      <c r="K25" s="48"/>
+      <c r="L25" s="48"/>
+      <c r="M25" s="48"/>
+      <c r="N25" s="48"/>
+      <c r="O25" s="48"/>
+      <c r="P25" s="48"/>
+      <c r="Q25" s="48"/>
+      <c r="R25" s="48"/>
+      <c r="S25" s="49"/>
+    </row>
+    <row r="26" spans="2:54" x14ac:dyDescent="0.25">
+      <c r="B26" s="50" t="s">
         <v>70</v>
       </c>
-      <c r="C22" s="51"/>
-      <c r="D22" s="51"/>
-      <c r="E22" s="51"/>
-      <c r="F22" s="51"/>
-      <c r="G22" s="51"/>
-      <c r="H22" s="51"/>
-      <c r="I22" s="51"/>
-      <c r="J22" s="51"/>
-      <c r="K22" s="51"/>
-      <c r="L22" s="51"/>
-      <c r="M22" s="51"/>
-      <c r="N22" s="51"/>
-      <c r="O22" s="51"/>
-      <c r="P22" s="51"/>
-      <c r="Q22" s="51"/>
-      <c r="R22" s="51"/>
-      <c r="S22" s="52"/>
+      <c r="C26" s="51"/>
+      <c r="D26" s="51"/>
+      <c r="E26" s="51"/>
+      <c r="F26" s="51"/>
+      <c r="G26" s="51"/>
+      <c r="H26" s="51"/>
+      <c r="I26" s="51"/>
+      <c r="J26" s="51"/>
+      <c r="K26" s="51"/>
+      <c r="L26" s="51"/>
+      <c r="M26" s="51"/>
+      <c r="N26" s="51"/>
+      <c r="O26" s="51"/>
+      <c r="P26" s="51"/>
+      <c r="Q26" s="51"/>
+      <c r="R26" s="51"/>
+      <c r="S26" s="52"/>
     </row>
   </sheetData>
-  <mergeCells count="22">
+  <mergeCells count="35">
+    <mergeCell ref="HV4:IX4"/>
     <mergeCell ref="X1:Y1"/>
-    <mergeCell ref="AR4:AR12"/>
-    <mergeCell ref="AS4:AV12"/>
-    <mergeCell ref="AZ4:AZ12"/>
-    <mergeCell ref="BB4:BB12"/>
-    <mergeCell ref="AY4:AY12"/>
-    <mergeCell ref="AJ13:BB13"/>
-    <mergeCell ref="B16:S16"/>
-    <mergeCell ref="H4:S4"/>
-    <mergeCell ref="H7:S7"/>
-    <mergeCell ref="H6:S6"/>
-    <mergeCell ref="AJ4:AJ12"/>
-    <mergeCell ref="AK4:AK12"/>
-    <mergeCell ref="AL4:AQ12"/>
-    <mergeCell ref="H12:S12"/>
+    <mergeCell ref="AR8:AR16"/>
+    <mergeCell ref="AS8:AV16"/>
+    <mergeCell ref="AZ8:AZ16"/>
+    <mergeCell ref="BB8:BB16"/>
+    <mergeCell ref="AY8:AY16"/>
+    <mergeCell ref="AL1:AQ1"/>
+    <mergeCell ref="AJ17:BB17"/>
+    <mergeCell ref="B20:S20"/>
+    <mergeCell ref="H8:S8"/>
     <mergeCell ref="H11:S11"/>
     <mergeCell ref="H10:S10"/>
+    <mergeCell ref="AJ8:AJ16"/>
+    <mergeCell ref="AK8:AK16"/>
+    <mergeCell ref="AL8:AQ16"/>
+    <mergeCell ref="H16:S16"/>
+    <mergeCell ref="H15:S15"/>
+    <mergeCell ref="H14:S14"/>
+    <mergeCell ref="H13:S13"/>
+    <mergeCell ref="H12:S12"/>
     <mergeCell ref="H9:S9"/>
-    <mergeCell ref="H8:S8"/>
-    <mergeCell ref="H5:S5"/>
-    <mergeCell ref="H13:S13"/>
-    <mergeCell ref="H14:S14"/>
+    <mergeCell ref="H17:S17"/>
+    <mergeCell ref="H18:S18"/>
+    <mergeCell ref="BE1:BJ1"/>
+    <mergeCell ref="BX1:CC1"/>
+    <mergeCell ref="CQ1:CV1"/>
+    <mergeCell ref="DJ1:DO1"/>
+    <mergeCell ref="EA1:EF1"/>
+    <mergeCell ref="HY1:IJ1"/>
+    <mergeCell ref="ER1:EW1"/>
+    <mergeCell ref="FI1:FN1"/>
+    <mergeCell ref="FZ1:GE1"/>
+    <mergeCell ref="GQ1:GV1"/>
+    <mergeCell ref="HH1:HM1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>